<commit_message>
feat: pre-populate process types in shortage inquiry and enhance admin interface for sign-off status
</commit_message>
<xml_diff>
--- a/Newdata/半品未撥.XLSX
+++ b/Newdata/半品未撥.XLSX
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="191">
   <si>
     <t>ZP02</t>
   </si>
@@ -469,6 +469,51 @@
     <t>200006700</t>
   </si>
   <si>
+    <t>200006701</t>
+  </si>
+  <si>
+    <t>080200547500</t>
+  </si>
+  <si>
+    <t>MVP13機頭D15K,011237_#40,38F18</t>
+  </si>
+  <si>
+    <t>200006702</t>
+  </si>
+  <si>
+    <t>200006703</t>
+  </si>
+  <si>
+    <t>080200422904</t>
+  </si>
+  <si>
+    <t>HEP機頭G8K,011194_780,55A18,C</t>
+  </si>
+  <si>
+    <t>200006704</t>
+  </si>
+  <si>
+    <t>200006705</t>
+  </si>
+  <si>
+    <t>080100037203</t>
+  </si>
+  <si>
+    <t>D8K 主軸,021274_BT50,M50,C045</t>
+  </si>
+  <si>
+    <t>200006706</t>
+  </si>
+  <si>
+    <t>200006707</t>
+  </si>
+  <si>
+    <t>080100045603</t>
+  </si>
+  <si>
+    <t>D12K 主軸,021274_BBT50,M50,CW45</t>
+  </si>
+  <si>
     <t>ZP09</t>
   </si>
   <si>
@@ -482,6 +527,15 @@
   </si>
   <si>
     <t>PENNY</t>
+  </si>
+  <si>
+    <t>630000355</t>
+  </si>
+  <si>
+    <t>080100145601</t>
+  </si>
+  <si>
+    <t>D6K 主軸,010801_BT50,M50E,0045</t>
   </si>
   <si>
     <t>訂單類型</t>
@@ -634,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="6" customWidth="1"/>
@@ -657,52 +711,52 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -4357,51 +4411,451 @@
     </row>
     <row r="75" spans="1:16">
       <c r="A75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B75" t="s">
         <v>152</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" s="2">
+        <v>1</v>
+      </c>
+      <c r="D75" s="2">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
         <v>153</v>
       </c>
-      <c r="C75" s="2">
-        <v>1</v>
-      </c>
-      <c r="D75" s="2">
-        <v>0</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>154</v>
       </c>
-      <c r="F75" t="s">
+      <c r="G75" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H75" s="3">
+        <v>46140</v>
+      </c>
+      <c r="I75" s="3">
+        <v>46142</v>
+      </c>
+      <c r="J75" t="s">
+        <v>4</v>
+      </c>
+      <c r="K75" t="s">
+        <v>5</v>
+      </c>
+      <c r="L75" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M75" t="s">
+        <v>6</v>
+      </c>
+      <c r="N75" t="s">
+        <v>7</v>
+      </c>
+      <c r="O75" t="s">
+        <v>8</v>
+      </c>
+      <c r="P75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
         <v>155</v>
       </c>
-      <c r="G75" s="3">
+      <c r="C76" s="2">
+        <v>1</v>
+      </c>
+      <c r="D76" s="2">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>71</v>
+      </c>
+      <c r="F76" t="s">
+        <v>72</v>
+      </c>
+      <c r="G76" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H76" s="3">
+        <v>46140</v>
+      </c>
+      <c r="I76" s="3">
+        <v>46146</v>
+      </c>
+      <c r="J76" t="s">
+        <v>11</v>
+      </c>
+      <c r="K76" t="s">
+        <v>5</v>
+      </c>
+      <c r="L76" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M76" t="s">
+        <v>6</v>
+      </c>
+      <c r="N76" t="s">
+        <v>7</v>
+      </c>
+      <c r="O76" t="s">
+        <v>8</v>
+      </c>
+      <c r="P76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16">
+      <c r="A77" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" t="s">
+        <v>156</v>
+      </c>
+      <c r="C77" s="2">
+        <v>1</v>
+      </c>
+      <c r="D77" s="2">
+        <v>0</v>
+      </c>
+      <c r="E77" t="s">
+        <v>157</v>
+      </c>
+      <c r="F77" t="s">
+        <v>158</v>
+      </c>
+      <c r="G77" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H77" s="3">
+        <v>46183</v>
+      </c>
+      <c r="I77" s="3">
+        <v>46190</v>
+      </c>
+      <c r="J77" t="s">
+        <v>65</v>
+      </c>
+      <c r="K77" t="s">
+        <v>5</v>
+      </c>
+      <c r="L77" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M77" t="s">
+        <v>6</v>
+      </c>
+      <c r="N77" t="s">
+        <v>7</v>
+      </c>
+      <c r="O77" t="s">
+        <v>8</v>
+      </c>
+      <c r="P77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" t="s">
+        <v>159</v>
+      </c>
+      <c r="C78" s="2">
+        <v>1</v>
+      </c>
+      <c r="D78" s="2">
+        <v>0</v>
+      </c>
+      <c r="E78" t="s">
+        <v>157</v>
+      </c>
+      <c r="F78" t="s">
+        <v>158</v>
+      </c>
+      <c r="G78" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H78" s="3">
+        <v>46183</v>
+      </c>
+      <c r="I78" s="3">
+        <v>46190</v>
+      </c>
+      <c r="J78" t="s">
+        <v>81</v>
+      </c>
+      <c r="K78" t="s">
+        <v>5</v>
+      </c>
+      <c r="L78" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M78" t="s">
+        <v>6</v>
+      </c>
+      <c r="N78" t="s">
+        <v>7</v>
+      </c>
+      <c r="O78" t="s">
+        <v>8</v>
+      </c>
+      <c r="P78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16">
+      <c r="A79" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" t="s">
+        <v>160</v>
+      </c>
+      <c r="C79" s="2">
+        <v>1</v>
+      </c>
+      <c r="D79" s="2">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>161</v>
+      </c>
+      <c r="F79" t="s">
+        <v>162</v>
+      </c>
+      <c r="G79" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H79" s="3">
+        <v>46176</v>
+      </c>
+      <c r="I79" s="3">
+        <v>46182</v>
+      </c>
+      <c r="J79" t="s">
+        <v>11</v>
+      </c>
+      <c r="K79" t="s">
+        <v>5</v>
+      </c>
+      <c r="L79" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M79" t="s">
+        <v>6</v>
+      </c>
+      <c r="N79" t="s">
+        <v>7</v>
+      </c>
+      <c r="O79" t="s">
+        <v>8</v>
+      </c>
+      <c r="P79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" t="s">
+        <v>163</v>
+      </c>
+      <c r="C80" s="2">
+        <v>1</v>
+      </c>
+      <c r="D80" s="2">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>161</v>
+      </c>
+      <c r="F80" t="s">
+        <v>162</v>
+      </c>
+      <c r="G80" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H80" s="3">
+        <v>46176</v>
+      </c>
+      <c r="I80" s="3">
+        <v>46182</v>
+      </c>
+      <c r="J80" t="s">
+        <v>81</v>
+      </c>
+      <c r="K80" t="s">
+        <v>5</v>
+      </c>
+      <c r="L80" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M80" t="s">
+        <v>6</v>
+      </c>
+      <c r="N80" t="s">
+        <v>7</v>
+      </c>
+      <c r="O80" t="s">
+        <v>8</v>
+      </c>
+      <c r="P80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16">
+      <c r="A81" t="s">
+        <v>0</v>
+      </c>
+      <c r="B81" t="s">
+        <v>164</v>
+      </c>
+      <c r="C81" s="2">
+        <v>1</v>
+      </c>
+      <c r="D81" s="2">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>165</v>
+      </c>
+      <c r="F81" t="s">
+        <v>166</v>
+      </c>
+      <c r="G81" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H81" s="3">
+        <v>46140</v>
+      </c>
+      <c r="I81" s="3">
+        <v>46147</v>
+      </c>
+      <c r="J81" t="s">
+        <v>11</v>
+      </c>
+      <c r="K81" t="s">
+        <v>5</v>
+      </c>
+      <c r="L81" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M81" t="s">
+        <v>6</v>
+      </c>
+      <c r="N81" t="s">
+        <v>7</v>
+      </c>
+      <c r="O81" t="s">
+        <v>8</v>
+      </c>
+      <c r="P81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16">
+      <c r="A82" t="s">
+        <v>167</v>
+      </c>
+      <c r="B82" t="s">
+        <v>168</v>
+      </c>
+      <c r="C82" s="2">
+        <v>1</v>
+      </c>
+      <c r="D82" s="2">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>169</v>
+      </c>
+      <c r="F82" t="s">
+        <v>170</v>
+      </c>
+      <c r="G82" s="3">
         <v>46043</v>
       </c>
-      <c r="H75" s="3">
+      <c r="H82" s="3">
         <v>46051</v>
       </c>
-      <c r="I75" s="3">
+      <c r="I82" s="3">
         <v>46057</v>
       </c>
-      <c r="J75" t="s">
+      <c r="J82" t="s">
         <v>11</v>
       </c>
-      <c r="K75" t="s">
-        <v>156</v>
-      </c>
-      <c r="L75" s="3">
+      <c r="K82" t="s">
+        <v>171</v>
+      </c>
+      <c r="L82" s="3">
         <v>46043</v>
       </c>
-      <c r="M75" t="s">
-        <v>6</v>
-      </c>
-      <c r="N75" t="s">
-        <v>7</v>
-      </c>
-      <c r="O75" t="s">
-        <v>8</v>
-      </c>
-      <c r="P75" t="s">
+      <c r="M82" t="s">
+        <v>6</v>
+      </c>
+      <c r="N82" t="s">
+        <v>7</v>
+      </c>
+      <c r="O82" t="s">
+        <v>8</v>
+      </c>
+      <c r="P82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16">
+      <c r="A83" t="s">
+        <v>167</v>
+      </c>
+      <c r="B83" t="s">
+        <v>172</v>
+      </c>
+      <c r="C83" s="2">
+        <v>1</v>
+      </c>
+      <c r="D83" s="2">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>173</v>
+      </c>
+      <c r="F83" t="s">
+        <v>174</v>
+      </c>
+      <c r="G83" s="3">
+        <v>46140</v>
+      </c>
+      <c r="H83" s="3">
+        <v>46140</v>
+      </c>
+      <c r="I83" s="3">
+        <v>46147</v>
+      </c>
+      <c r="J83" t="s">
+        <v>11</v>
+      </c>
+      <c r="K83" t="s">
+        <v>171</v>
+      </c>
+      <c r="L83" s="3">
+        <v>46140</v>
+      </c>
+      <c r="M83" t="s">
+        <v>6</v>
+      </c>
+      <c r="N83" t="s">
+        <v>7</v>
+      </c>
+      <c r="O83" t="s">
+        <v>8</v>
+      </c>
+      <c r="P83" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix material sorting and implement auto-dispatch for semi-finished goods
</commit_message>
<xml_diff>
--- a/Newdata/半品未撥.XLSX
+++ b/Newdata/半品未撥.XLSX
@@ -11,12 +11,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="203">
   <si>
     <t>ZP02</t>
   </si>
   <si>
-    <t>200006507</t>
+    <t>200006512</t>
+  </si>
+  <si>
+    <t>080200538802</t>
+  </si>
+  <si>
+    <t>H1682機頭G6K,021314_#50,55F23,C</t>
+  </si>
+  <si>
+    <t>REL  PRC  MANC SETC</t>
+  </si>
+  <si>
+    <t>SDCHANG</t>
+  </si>
+  <si>
+    <t>SHEO</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>200006513</t>
+  </si>
+  <si>
+    <t>200006514</t>
+  </si>
+  <si>
+    <t>200006516</t>
+  </si>
+  <si>
+    <t>080100116405</t>
+  </si>
+  <si>
+    <t>G6K 主軸,021305_BBT50,CW45</t>
+  </si>
+  <si>
+    <t>200006517</t>
+  </si>
+  <si>
+    <t>200006518</t>
+  </si>
+  <si>
+    <t>200006519</t>
   </si>
   <si>
     <t>080200545001</t>
@@ -25,99 +73,39 @@
     <t>H1370機頭G6K,011395_#50,55F23,C</t>
   </si>
   <si>
+    <t>200006520</t>
+  </si>
+  <si>
+    <t>200006521</t>
+  </si>
+  <si>
+    <t>200006522</t>
+  </si>
+  <si>
+    <t>200006537</t>
+  </si>
+  <si>
+    <t>080200546703</t>
+  </si>
+  <si>
+    <t>MVP11機頭D15K,031859_#40,38F18,C,AT8</t>
+  </si>
+  <si>
+    <t>200006538</t>
+  </si>
+  <si>
+    <t>200006539</t>
+  </si>
+  <si>
+    <t>080100156608</t>
+  </si>
+  <si>
+    <t>DA15K 主軸,021857_BBT40,M60,CW45</t>
+  </si>
+  <si>
     <t>REL  PRC  MACM SETC</t>
   </si>
   <si>
-    <t>SDCHANG</t>
-  </si>
-  <si>
-    <t>SHEO</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>200006508</t>
-  </si>
-  <si>
-    <t>REL  PRC  MANC SETC</t>
-  </si>
-  <si>
-    <t>200006509</t>
-  </si>
-  <si>
-    <t>080100116405</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021305_BBT50,CW45</t>
-  </si>
-  <si>
-    <t>200006510</t>
-  </si>
-  <si>
-    <t>200006512</t>
-  </si>
-  <si>
-    <t>080200538802</t>
-  </si>
-  <si>
-    <t>H1682機頭G6K,021314_#50,55F23,C</t>
-  </si>
-  <si>
-    <t>200006513</t>
-  </si>
-  <si>
-    <t>200006514</t>
-  </si>
-  <si>
-    <t>200006516</t>
-  </si>
-  <si>
-    <t>200006517</t>
-  </si>
-  <si>
-    <t>200006518</t>
-  </si>
-  <si>
-    <t>200006519</t>
-  </si>
-  <si>
-    <t>200006520</t>
-  </si>
-  <si>
-    <t>200006521</t>
-  </si>
-  <si>
-    <t>200006522</t>
-  </si>
-  <si>
-    <t>200006537</t>
-  </si>
-  <si>
-    <t>080200546703</t>
-  </si>
-  <si>
-    <t>MVP11機頭D15K,031859_#40,38F18,C,AT8</t>
-  </si>
-  <si>
-    <t>200006538</t>
-  </si>
-  <si>
-    <t>200006539</t>
-  </si>
-  <si>
-    <t>080100156608</t>
-  </si>
-  <si>
-    <t>DA15K 主軸,021857_BBT40,M60,CW45</t>
-  </si>
-  <si>
     <t>200006540</t>
   </si>
   <si>
@@ -133,15 +121,6 @@
     <t>200006544</t>
   </si>
   <si>
-    <t>200006554</t>
-  </si>
-  <si>
-    <t>080200037902</t>
-  </si>
-  <si>
-    <t>HSA機頭G6K,021563_1200,BBT50,55,045</t>
-  </si>
-  <si>
     <t>200006567</t>
   </si>
   <si>
@@ -160,18 +139,6 @@
     <t>自動頭HF-AU,031911_2.5°-BBT50-45°-4K-C-F</t>
   </si>
   <si>
-    <t>200006569</t>
-  </si>
-  <si>
-    <t>080300030000</t>
-  </si>
-  <si>
-    <t>自動頭HF-AU,032731,G5K_1°-BT50-DIN-5K-C-F</t>
-  </si>
-  <si>
-    <t>REL  MSPT PCNF PRC  MANC SETC</t>
-  </si>
-  <si>
     <t>200006575</t>
   </si>
   <si>
@@ -391,7 +358,25 @@
     <t>200006685</t>
   </si>
   <si>
-    <t>200006687</t>
+    <t>200006693</t>
+  </si>
+  <si>
+    <t>080200538702</t>
+  </si>
+  <si>
+    <t>H1682機頭G6K,021314_#50,48F23,C</t>
+  </si>
+  <si>
+    <t>200006694</t>
+  </si>
+  <si>
+    <t>200006695</t>
+  </si>
+  <si>
+    <t>200006696</t>
+  </si>
+  <si>
+    <t>200006697</t>
   </si>
   <si>
     <t>080200538402</t>
@@ -400,54 +385,6 @@
     <t>H1682機頭G6K,021314_#50,48F23,0</t>
   </si>
   <si>
-    <t>200006688</t>
-  </si>
-  <si>
-    <t>080100112405</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021305_BT50,0W45</t>
-  </si>
-  <si>
-    <t>200006689</t>
-  </si>
-  <si>
-    <t>080100113205</t>
-  </si>
-  <si>
-    <t>G6K 主軸,021305_BT50,CW45</t>
-  </si>
-  <si>
-    <t>200006690</t>
-  </si>
-  <si>
-    <t>200006691</t>
-  </si>
-  <si>
-    <t>200006692</t>
-  </si>
-  <si>
-    <t>200006693</t>
-  </si>
-  <si>
-    <t>080200538702</t>
-  </si>
-  <si>
-    <t>H1682機頭G6K,021314_#50,48F23,C</t>
-  </si>
-  <si>
-    <t>200006694</t>
-  </si>
-  <si>
-    <t>200006695</t>
-  </si>
-  <si>
-    <t>200006696</t>
-  </si>
-  <si>
-    <t>200006697</t>
-  </si>
-  <si>
     <t>200006698</t>
   </si>
   <si>
@@ -466,21 +403,6 @@
     <t>D20K 主軸,010683_A63,M50,CW</t>
   </si>
   <si>
-    <t>200006700</t>
-  </si>
-  <si>
-    <t>200006701</t>
-  </si>
-  <si>
-    <t>080200547500</t>
-  </si>
-  <si>
-    <t>MVP13機頭D15K,011237_#40,38F18</t>
-  </si>
-  <si>
-    <t>200006702</t>
-  </si>
-  <si>
     <t>200006703</t>
   </si>
   <si>
@@ -505,13 +427,136 @@
     <t>200006706</t>
   </si>
   <si>
-    <t>200006707</t>
-  </si>
-  <si>
-    <t>080100045603</t>
-  </si>
-  <si>
-    <t>D12K 主軸,021274_BBT50,M50,CW45</t>
+    <t>200006708</t>
+  </si>
+  <si>
+    <t>080200546502</t>
+  </si>
+  <si>
+    <t>MVP11機頭D15K,031859_#40,32F18,0</t>
+  </si>
+  <si>
+    <t>200006709</t>
+  </si>
+  <si>
+    <t>200006710</t>
+  </si>
+  <si>
+    <t>200006711</t>
+  </si>
+  <si>
+    <t>200006712</t>
+  </si>
+  <si>
+    <t>200006713</t>
+  </si>
+  <si>
+    <t>200006714</t>
+  </si>
+  <si>
+    <t>200006715</t>
+  </si>
+  <si>
+    <t>200006716</t>
+  </si>
+  <si>
+    <t>200006717</t>
+  </si>
+  <si>
+    <t>200006718</t>
+  </si>
+  <si>
+    <t>200006719</t>
+  </si>
+  <si>
+    <t>200006720</t>
+  </si>
+  <si>
+    <t>080200551400</t>
+  </si>
+  <si>
+    <t>SP10機頭P12K,021023_#40,5GT-72,C</t>
+  </si>
+  <si>
+    <t>200006721</t>
+  </si>
+  <si>
+    <t>080200095202</t>
+  </si>
+  <si>
+    <t>HSA機頭G8K,011147_1000,55A22,C</t>
+  </si>
+  <si>
+    <t>200006722</t>
+  </si>
+  <si>
+    <t>080100048401</t>
+  </si>
+  <si>
+    <t>G8K 主軸,011119_BBT50,M50,C045</t>
+  </si>
+  <si>
+    <t>200006723</t>
+  </si>
+  <si>
+    <t>080200026005</t>
+  </si>
+  <si>
+    <t>PBM135機頭G2.5K,010831_BT50,MO1C45</t>
+  </si>
+  <si>
+    <t>200006724</t>
+  </si>
+  <si>
+    <t>080100033603</t>
+  </si>
+  <si>
+    <t>G2.5K主軸,010830_BT50,C045</t>
+  </si>
+  <si>
+    <t>200006725</t>
+  </si>
+  <si>
+    <t>080200483300</t>
+  </si>
+  <si>
+    <t>H1365機頭G8K,021863_#40,42F25,C</t>
+  </si>
+  <si>
+    <t>200006726</t>
+  </si>
+  <si>
+    <t>080100108701</t>
+  </si>
+  <si>
+    <t>G8K 主軸,021534_BT40,CWDIN</t>
+  </si>
+  <si>
+    <t>200006727</t>
+  </si>
+  <si>
+    <t>080200563000</t>
+  </si>
+  <si>
+    <t>LG1370NEO機頭P12K,021964_#40,8YU-84,C</t>
+  </si>
+  <si>
+    <t>200006728</t>
+  </si>
+  <si>
+    <t>080100076704</t>
+  </si>
+  <si>
+    <t>P12K 主軸,021444_BT40,8YU,CWDIN</t>
+  </si>
+  <si>
+    <t>200006729</t>
+  </si>
+  <si>
+    <t>080200572200</t>
+  </si>
+  <si>
+    <t>L2100機頭D12K,021634_#40,48F23</t>
   </si>
   <si>
     <t>ZP09</t>
@@ -527,15 +572,6 @@
   </si>
   <si>
     <t>PENNY</t>
-  </si>
-  <si>
-    <t>630000355</t>
-  </si>
-  <si>
-    <t>080100145601</t>
-  </si>
-  <si>
-    <t>D6K 主軸,010801_BT50,M50E,0045</t>
   </si>
   <si>
     <t>訂單類型</t>
@@ -688,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="6" customWidth="1"/>
@@ -696,11 +732,11 @@
     <col min="3" max="3" bestFit="1" width="9" customWidth="1"/>
     <col min="4" max="4" bestFit="1" width="9" customWidth="1"/>
     <col min="5" max="5" bestFit="1" width="14" customWidth="1"/>
-    <col min="6" max="6" bestFit="1" width="40" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="39" customWidth="1"/>
     <col min="7" max="7" bestFit="1" width="13" customWidth="1"/>
     <col min="8" max="8" bestFit="1" width="13" customWidth="1"/>
     <col min="9" max="9" bestFit="1" width="13" customWidth="1"/>
-    <col min="10" max="10" bestFit="1" width="31" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="26" customWidth="1"/>
     <col min="11" max="11" bestFit="1" width="9" customWidth="1"/>
     <col min="12" max="12" bestFit="1" width="13" customWidth="1"/>
     <col min="13" max="13" bestFit="1" width="8" customWidth="1"/>
@@ -711,52 +747,52 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -782,10 +818,10 @@
         <v>46064</v>
       </c>
       <c r="H2" s="3">
-        <v>46240</v>
+        <v>46174</v>
       </c>
       <c r="I2" s="3">
-        <v>46245</v>
+        <v>46177</v>
       </c>
       <c r="J2" t="s">
         <v>4</v>
@@ -832,13 +868,13 @@
         <v>46064</v>
       </c>
       <c r="H3" s="3">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="I3" s="3">
-        <v>46245</v>
+        <v>46241</v>
       </c>
       <c r="J3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K3" t="s">
         <v>5</v>
@@ -864,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
@@ -873,19 +909,19 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G4" s="3">
         <v>46064</v>
       </c>
       <c r="H4" s="3">
-        <v>46234</v>
+        <v>46297</v>
       </c>
       <c r="I4" s="3">
-        <v>46239</v>
+        <v>46302</v>
       </c>
       <c r="J4" t="s">
         <v>4</v>
@@ -914,7 +950,7 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
@@ -932,13 +968,13 @@
         <v>46064</v>
       </c>
       <c r="H5" s="3">
-        <v>46234</v>
+        <v>46168</v>
       </c>
       <c r="I5" s="3">
-        <v>46239</v>
+        <v>46171</v>
       </c>
       <c r="J5" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K5" t="s">
         <v>5</v>
@@ -964,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
@@ -973,22 +1009,22 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G6" s="3">
         <v>46064</v>
       </c>
       <c r="H6" s="3">
-        <v>46174</v>
+        <v>46232</v>
       </c>
       <c r="I6" s="3">
-        <v>46177</v>
+        <v>46237</v>
       </c>
       <c r="J6" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K6" t="s">
         <v>5</v>
@@ -1014,7 +1050,7 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -1023,22 +1059,22 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G7" s="3">
         <v>46064</v>
       </c>
       <c r="H7" s="3">
-        <v>46238</v>
+        <v>46289</v>
       </c>
       <c r="I7" s="3">
-        <v>46241</v>
+        <v>46296</v>
       </c>
       <c r="J7" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K7" t="s">
         <v>5</v>
@@ -1064,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
@@ -1073,22 +1109,22 @@
         <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G8" s="3">
-        <v>46064</v>
+        <v>46090</v>
       </c>
       <c r="H8" s="3">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="I8" s="3">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="J8" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K8" t="s">
         <v>5</v>
@@ -1114,7 +1150,7 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
@@ -1123,22 +1159,22 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G9" s="3">
         <v>46064</v>
       </c>
       <c r="H9" s="3">
-        <v>46168</v>
+        <v>46301</v>
       </c>
       <c r="I9" s="3">
-        <v>46171</v>
+        <v>46307</v>
       </c>
       <c r="J9" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K9" t="s">
         <v>5</v>
@@ -1164,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2">
         <v>1</v>
@@ -1182,13 +1218,13 @@
         <v>46064</v>
       </c>
       <c r="H10" s="3">
-        <v>46232</v>
+        <v>46267</v>
       </c>
       <c r="I10" s="3">
-        <v>46237</v>
+        <v>46272</v>
       </c>
       <c r="J10" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K10" t="s">
         <v>5</v>
@@ -1214,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
@@ -1232,13 +1268,13 @@
         <v>46064</v>
       </c>
       <c r="H11" s="3">
-        <v>46289</v>
+        <v>46267</v>
       </c>
       <c r="I11" s="3">
-        <v>46296</v>
+        <v>46272</v>
       </c>
       <c r="J11" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K11" t="s">
         <v>5</v>
@@ -1264,37 +1300,37 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="2">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" t="s">
-        <v>2</v>
-      </c>
       <c r="F12" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G12" s="3">
-        <v>46090</v>
+        <v>46076</v>
       </c>
       <c r="H12" s="3">
-        <v>46301</v>
+        <v>46212</v>
       </c>
       <c r="I12" s="3">
-        <v>46307</v>
+        <v>46216</v>
       </c>
       <c r="J12" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K12" t="s">
         <v>5</v>
       </c>
       <c r="L12" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="M12" t="s">
         <v>6</v>
@@ -1314,37 +1350,37 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="2">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="E13" t="s">
-        <v>2</v>
-      </c>
-      <c r="F13" t="s">
-        <v>3</v>
-      </c>
       <c r="G13" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="H13" s="3">
-        <v>46301</v>
+        <v>46212</v>
       </c>
       <c r="I13" s="3">
-        <v>46307</v>
+        <v>46216</v>
       </c>
       <c r="J13" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K13" t="s">
         <v>5</v>
       </c>
       <c r="L13" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="M13" t="s">
         <v>6</v>
@@ -1364,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="2">
         <v>1</v>
@@ -1373,28 +1409,28 @@
         <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G14" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="H14" s="3">
-        <v>46267</v>
+        <v>46206</v>
       </c>
       <c r="I14" s="3">
-        <v>46272</v>
+        <v>46211</v>
       </c>
       <c r="J14" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K14" t="s">
         <v>5</v>
       </c>
       <c r="L14" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="M14" t="s">
         <v>6</v>
@@ -1414,7 +1450,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -1423,28 +1459,28 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G15" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="H15" s="3">
-        <v>46267</v>
+        <v>46206</v>
       </c>
       <c r="I15" s="3">
-        <v>46272</v>
+        <v>46211</v>
       </c>
       <c r="J15" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K15" t="s">
         <v>5</v>
       </c>
       <c r="L15" s="3">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="M15" t="s">
         <v>6</v>
@@ -1464,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -1473,22 +1509,22 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G16" s="3">
         <v>46076</v>
       </c>
       <c r="H16" s="3">
-        <v>46212</v>
+        <v>46251</v>
       </c>
       <c r="I16" s="3">
-        <v>46216</v>
+        <v>46253</v>
       </c>
       <c r="J16" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K16" t="s">
         <v>5</v>
@@ -1514,7 +1550,7 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C17" s="2">
         <v>1</v>
@@ -1523,22 +1559,22 @@
         <v>0</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G17" s="3">
         <v>46076</v>
       </c>
       <c r="H17" s="3">
-        <v>46212</v>
+        <v>46251</v>
       </c>
       <c r="I17" s="3">
-        <v>46216</v>
+        <v>46253</v>
       </c>
       <c r="J17" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K17" t="s">
         <v>5</v>
@@ -1564,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -1573,22 +1609,22 @@
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F18" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G18" s="3">
         <v>46076</v>
       </c>
       <c r="H18" s="3">
-        <v>46206</v>
+        <v>46245</v>
       </c>
       <c r="I18" s="3">
-        <v>46211</v>
+        <v>46248</v>
       </c>
       <c r="J18" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K18" t="s">
         <v>5</v>
@@ -1623,22 +1659,22 @@
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F19" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G19" s="3">
         <v>46076</v>
       </c>
       <c r="H19" s="3">
-        <v>46206</v>
+        <v>46245</v>
       </c>
       <c r="I19" s="3">
-        <v>46211</v>
+        <v>46248</v>
       </c>
       <c r="J19" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K19" t="s">
         <v>5</v>
@@ -1673,28 +1709,28 @@
         <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G20" s="3">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="H20" s="3">
-        <v>46251</v>
+        <v>46148</v>
       </c>
       <c r="I20" s="3">
-        <v>46253</v>
+        <v>46171</v>
       </c>
       <c r="J20" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K20" t="s">
         <v>5</v>
       </c>
       <c r="L20" s="3">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="M20" t="s">
         <v>6</v>
@@ -1714,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C21" s="2">
         <v>1</v>
@@ -1723,28 +1759,28 @@
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G21" s="3">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="H21" s="3">
-        <v>46251</v>
+        <v>46148</v>
       </c>
       <c r="I21" s="3">
-        <v>46253</v>
+        <v>46171</v>
       </c>
       <c r="J21" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K21" t="s">
         <v>5</v>
       </c>
       <c r="L21" s="3">
-        <v>46076</v>
+        <v>46083</v>
       </c>
       <c r="M21" t="s">
         <v>6</v>
@@ -1764,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -1773,19 +1809,19 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F22" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G22" s="3">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="H22" s="3">
-        <v>46245</v>
+        <v>46167</v>
       </c>
       <c r="I22" s="3">
-        <v>46248</v>
+        <v>46185</v>
       </c>
       <c r="J22" t="s">
         <v>4</v>
@@ -1794,7 +1830,7 @@
         <v>5</v>
       </c>
       <c r="L22" s="3">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="M22" t="s">
         <v>6</v>
@@ -1814,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C23" s="2">
         <v>1</v>
@@ -1823,28 +1859,28 @@
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G23" s="3">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="H23" s="3">
-        <v>46245</v>
+        <v>46213</v>
       </c>
       <c r="I23" s="3">
-        <v>46248</v>
+        <v>46217</v>
       </c>
       <c r="J23" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K23" t="s">
         <v>5</v>
       </c>
       <c r="L23" s="3">
-        <v>46076</v>
+        <v>46086</v>
       </c>
       <c r="M23" t="s">
         <v>6</v>
@@ -1864,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C24" s="2">
         <v>1</v>
@@ -1873,28 +1909,28 @@
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G24" s="3">
-        <v>46079</v>
+        <v>46086</v>
       </c>
       <c r="H24" s="3">
-        <v>46155</v>
+        <v>46191</v>
       </c>
       <c r="I24" s="3">
-        <v>46160</v>
+        <v>46210</v>
       </c>
       <c r="J24" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K24" t="s">
         <v>5</v>
       </c>
       <c r="L24" s="3">
-        <v>46079</v>
+        <v>46086</v>
       </c>
       <c r="M24" t="s">
         <v>6</v>
@@ -1914,7 +1950,7 @@
         <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -1923,28 +1959,28 @@
         <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="F25" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="G25" s="3">
-        <v>46083</v>
+        <v>46090</v>
       </c>
       <c r="H25" s="3">
-        <v>46148</v>
+        <v>46170</v>
       </c>
       <c r="I25" s="3">
-        <v>46171</v>
+        <v>46175</v>
       </c>
       <c r="J25" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="K25" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L25" s="3">
-        <v>46083</v>
+        <v>46090</v>
       </c>
       <c r="M25" t="s">
         <v>6</v>
@@ -1964,7 +2000,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -1973,28 +2009,28 @@
         <v>0</v>
       </c>
       <c r="E26" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="F26" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G26" s="3">
-        <v>46083</v>
+        <v>46090</v>
       </c>
       <c r="H26" s="3">
-        <v>46148</v>
+        <v>46206</v>
       </c>
       <c r="I26" s="3">
-        <v>46171</v>
+        <v>46210</v>
       </c>
       <c r="J26" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K26" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L26" s="3">
-        <v>46083</v>
+        <v>46090</v>
       </c>
       <c r="M26" t="s">
         <v>6</v>
@@ -2014,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
@@ -2023,28 +2059,28 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F27" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="G27" s="3">
-        <v>46084</v>
+        <v>46090</v>
       </c>
       <c r="H27" s="3">
-        <v>46135</v>
+        <v>46202</v>
       </c>
       <c r="I27" s="3">
-        <v>46157</v>
+        <v>46205</v>
       </c>
       <c r="J27" t="s">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="K27" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L27" s="3">
-        <v>46084</v>
+        <v>46090</v>
       </c>
       <c r="M27" t="s">
         <v>6</v>
@@ -2064,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
@@ -2073,28 +2109,28 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F28" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="G28" s="3">
-        <v>46086</v>
+        <v>46092</v>
       </c>
       <c r="H28" s="3">
-        <v>46167</v>
+        <v>46092</v>
       </c>
       <c r="I28" s="3">
-        <v>46185</v>
+        <v>46094</v>
       </c>
       <c r="J28" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K28" t="s">
         <v>5</v>
       </c>
       <c r="L28" s="3">
-        <v>46086</v>
+        <v>46092</v>
       </c>
       <c r="M28" t="s">
         <v>6</v>
@@ -2114,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C29" s="2">
         <v>1</v>
@@ -2123,19 +2159,19 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F29" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G29" s="3">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="H29" s="3">
-        <v>46213</v>
+        <v>46167</v>
       </c>
       <c r="I29" s="3">
-        <v>46217</v>
+        <v>46169</v>
       </c>
       <c r="J29" t="s">
         <v>4</v>
@@ -2144,7 +2180,7 @@
         <v>5</v>
       </c>
       <c r="L29" s="3">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="M29" t="s">
         <v>6</v>
@@ -2164,7 +2200,7 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C30" s="2">
         <v>1</v>
@@ -2173,19 +2209,19 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F30" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="G30" s="3">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="H30" s="3">
-        <v>46191</v>
+        <v>46167</v>
       </c>
       <c r="I30" s="3">
-        <v>46210</v>
+        <v>46169</v>
       </c>
       <c r="J30" t="s">
         <v>4</v>
@@ -2194,7 +2230,7 @@
         <v>5</v>
       </c>
       <c r="L30" s="3">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="M30" t="s">
         <v>6</v>
@@ -2214,7 +2250,7 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C31" s="2">
         <v>1</v>
@@ -2223,28 +2259,28 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F31" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G31" s="3">
-        <v>46090</v>
+        <v>46093</v>
       </c>
       <c r="H31" s="3">
-        <v>46170</v>
+        <v>46167</v>
       </c>
       <c r="I31" s="3">
-        <v>46175</v>
+        <v>46169</v>
       </c>
       <c r="J31" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="K31" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L31" s="3">
-        <v>46090</v>
+        <v>46093</v>
       </c>
       <c r="M31" t="s">
         <v>6</v>
@@ -2264,7 +2300,7 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
@@ -2273,28 +2309,28 @@
         <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="F32" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="G32" s="3">
-        <v>46090</v>
+        <v>46105</v>
       </c>
       <c r="H32" s="3">
-        <v>46206</v>
+        <v>46219</v>
       </c>
       <c r="I32" s="3">
-        <v>46210</v>
+        <v>46223</v>
       </c>
       <c r="J32" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K32" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L32" s="3">
-        <v>46090</v>
+        <v>46105</v>
       </c>
       <c r="M32" t="s">
         <v>6</v>
@@ -2314,7 +2350,7 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -2323,28 +2359,28 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F33" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G33" s="3">
-        <v>46090</v>
+        <v>46105</v>
       </c>
       <c r="H33" s="3">
-        <v>46202</v>
+        <v>46212</v>
       </c>
       <c r="I33" s="3">
-        <v>46205</v>
+        <v>46218</v>
       </c>
       <c r="J33" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K33" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L33" s="3">
-        <v>46090</v>
+        <v>46105</v>
       </c>
       <c r="M33" t="s">
         <v>6</v>
@@ -2364,7 +2400,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C34" s="2">
         <v>1</v>
@@ -2373,28 +2409,28 @@
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F34" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G34" s="3">
-        <v>46092</v>
+        <v>46106</v>
       </c>
       <c r="H34" s="3">
-        <v>46092</v>
+        <v>46227</v>
       </c>
       <c r="I34" s="3">
-        <v>46094</v>
+        <v>46231</v>
       </c>
       <c r="J34" t="s">
         <v>4</v>
       </c>
       <c r="K34" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L34" s="3">
-        <v>46092</v>
+        <v>46106</v>
       </c>
       <c r="M34" t="s">
         <v>6</v>
@@ -2414,7 +2450,7 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C35" s="2">
         <v>1</v>
@@ -2423,28 +2459,28 @@
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G35" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="H35" s="3">
-        <v>46167</v>
+        <v>46211</v>
       </c>
       <c r="I35" s="3">
-        <v>46169</v>
+        <v>46216</v>
       </c>
       <c r="J35" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K35" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L35" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="M35" t="s">
         <v>6</v>
@@ -2464,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
@@ -2473,28 +2509,28 @@
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F36" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="G36" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="H36" s="3">
-        <v>46167</v>
+        <v>46205</v>
       </c>
       <c r="I36" s="3">
-        <v>46169</v>
+        <v>46210</v>
       </c>
       <c r="J36" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K36" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L36" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="M36" t="s">
         <v>6</v>
@@ -2514,7 +2550,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C37" s="2">
         <v>1</v>
@@ -2523,28 +2559,28 @@
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="F37" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G37" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="H37" s="3">
-        <v>46167</v>
+        <v>46225</v>
       </c>
       <c r="I37" s="3">
-        <v>46169</v>
+        <v>46226</v>
       </c>
       <c r="J37" t="s">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="K37" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L37" s="3">
-        <v>46093</v>
+        <v>46106</v>
       </c>
       <c r="M37" t="s">
         <v>6</v>
@@ -2564,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2">
         <v>1</v>
@@ -2573,28 +2609,28 @@
         <v>0</v>
       </c>
       <c r="E38" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="F38" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="G38" s="3">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="H38" s="3">
         <v>46219</v>
       </c>
       <c r="I38" s="3">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="J38" t="s">
         <v>4</v>
       </c>
       <c r="K38" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L38" s="3">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="M38" t="s">
         <v>6</v>
@@ -2614,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C39" s="2">
         <v>1</v>
@@ -2623,28 +2659,28 @@
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F39" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G39" s="3">
-        <v>46105</v>
+        <v>46113</v>
       </c>
       <c r="H39" s="3">
-        <v>46212</v>
+        <v>46168</v>
       </c>
       <c r="I39" s="3">
-        <v>46218</v>
+        <v>46170</v>
       </c>
       <c r="J39" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K39" t="s">
         <v>5</v>
       </c>
       <c r="L39" s="3">
-        <v>46105</v>
+        <v>46113</v>
       </c>
       <c r="M39" t="s">
         <v>6</v>
@@ -2664,7 +2700,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C40" s="2">
         <v>1</v>
@@ -2673,28 +2709,28 @@
         <v>0</v>
       </c>
       <c r="E40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F40" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G40" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H40" s="3">
-        <v>46227</v>
+        <v>46168</v>
       </c>
       <c r="I40" s="3">
-        <v>46231</v>
+        <v>46170</v>
       </c>
       <c r="J40" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K40" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L40" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M40" t="s">
         <v>6</v>
@@ -2714,37 +2750,37 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="2">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
         <v>89</v>
       </c>
-      <c r="C41" s="2">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2">
-        <v>0</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>90</v>
       </c>
-      <c r="F41" t="s">
-        <v>91</v>
-      </c>
       <c r="G41" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H41" s="3">
-        <v>46211</v>
+        <v>46168</v>
       </c>
       <c r="I41" s="3">
-        <v>46216</v>
+        <v>46170</v>
       </c>
       <c r="J41" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K41" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L41" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M41" t="s">
         <v>6</v>
@@ -2764,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C42" s="2">
         <v>1</v>
@@ -2773,28 +2809,28 @@
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F42" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G42" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H42" s="3">
-        <v>46205</v>
+        <v>46232</v>
       </c>
       <c r="I42" s="3">
-        <v>46210</v>
+        <v>46234</v>
       </c>
       <c r="J42" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K42" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L42" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M42" t="s">
         <v>6</v>
@@ -2814,7 +2850,7 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C43" s="2">
         <v>1</v>
@@ -2823,28 +2859,28 @@
         <v>0</v>
       </c>
       <c r="E43" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F43" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="G43" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H43" s="3">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="I43" s="3">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="J43" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K43" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L43" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M43" t="s">
         <v>6</v>
@@ -2864,7 +2900,7 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C44" s="2">
         <v>1</v>
@@ -2873,28 +2909,28 @@
         <v>0</v>
       </c>
       <c r="E44" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="F44" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="G44" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H44" s="3">
-        <v>46219</v>
+        <v>46225</v>
       </c>
       <c r="I44" s="3">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="J44" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K44" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L44" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M44" t="s">
         <v>6</v>
@@ -2914,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C45" s="2">
         <v>1</v>
@@ -2923,22 +2959,22 @@
         <v>0</v>
       </c>
       <c r="E45" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F45" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G45" s="3">
         <v>46113</v>
       </c>
       <c r="H45" s="3">
-        <v>46168</v>
+        <v>46225</v>
       </c>
       <c r="I45" s="3">
-        <v>46170</v>
+        <v>46231</v>
       </c>
       <c r="J45" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K45" t="s">
         <v>5</v>
@@ -2964,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C46" s="2">
         <v>1</v>
@@ -2982,13 +3018,13 @@
         <v>46113</v>
       </c>
       <c r="H46" s="3">
-        <v>46168</v>
+        <v>46232</v>
       </c>
       <c r="I46" s="3">
-        <v>46170</v>
+        <v>46237</v>
       </c>
       <c r="J46" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K46" t="s">
         <v>5</v>
@@ -3014,31 +3050,31 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
+        <v>102</v>
+      </c>
+      <c r="C47" s="2">
+        <v>1</v>
+      </c>
+      <c r="D47" s="2">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="2">
-        <v>1</v>
-      </c>
-      <c r="D47" s="2">
-        <v>0</v>
-      </c>
-      <c r="E47" t="s">
-        <v>100</v>
-      </c>
       <c r="F47" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="G47" s="3">
         <v>46113</v>
       </c>
       <c r="H47" s="3">
-        <v>46168</v>
+        <v>46224</v>
       </c>
       <c r="I47" s="3">
-        <v>46170</v>
+        <v>46227</v>
       </c>
       <c r="J47" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K47" t="s">
         <v>5</v>
@@ -3073,28 +3109,28 @@
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F48" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G48" s="3">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="H48" s="3">
-        <v>46232</v>
+        <v>46149</v>
       </c>
       <c r="I48" s="3">
-        <v>46234</v>
+        <v>46153</v>
       </c>
       <c r="J48" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K48" t="s">
         <v>5</v>
       </c>
       <c r="L48" s="3">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="M48" t="s">
         <v>6</v>
@@ -3114,37 +3150,37 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
+        <v>107</v>
+      </c>
+      <c r="C49" s="2">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
         <v>105</v>
       </c>
-      <c r="C49" s="2">
-        <v>1</v>
-      </c>
-      <c r="D49" s="2">
-        <v>0</v>
-      </c>
-      <c r="E49" t="s">
-        <v>100</v>
-      </c>
       <c r="F49" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G49" s="3">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="H49" s="3">
-        <v>46232</v>
+        <v>46149</v>
       </c>
       <c r="I49" s="3">
-        <v>46234</v>
+        <v>46153</v>
       </c>
       <c r="J49" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K49" t="s">
         <v>5</v>
       </c>
       <c r="L49" s="3">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="M49" t="s">
         <v>6</v>
@@ -3164,7 +3200,7 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C50" s="2">
         <v>1</v>
@@ -3173,19 +3209,19 @@
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="F50" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="G50" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="H50" s="3">
-        <v>46225</v>
+        <v>46178</v>
       </c>
       <c r="I50" s="3">
-        <v>46231</v>
+        <v>46181</v>
       </c>
       <c r="J50" t="s">
         <v>4</v>
@@ -3194,7 +3230,7 @@
         <v>5</v>
       </c>
       <c r="L50" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="M50" t="s">
         <v>6</v>
@@ -3223,19 +3259,19 @@
         <v>0</v>
       </c>
       <c r="E51" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="F51" t="s">
-        <v>108</v>
+        <v>29</v>
       </c>
       <c r="G51" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="H51" s="3">
-        <v>46225</v>
+        <v>46174</v>
       </c>
       <c r="I51" s="3">
-        <v>46231</v>
+        <v>46177</v>
       </c>
       <c r="J51" t="s">
         <v>4</v>
@@ -3244,7 +3280,7 @@
         <v>5</v>
       </c>
       <c r="L51" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="M51" t="s">
         <v>6</v>
@@ -3279,22 +3315,22 @@
         <v>112</v>
       </c>
       <c r="G52" s="3">
-        <v>46113</v>
+        <v>46133</v>
       </c>
       <c r="H52" s="3">
-        <v>46232</v>
+        <v>46170</v>
       </c>
       <c r="I52" s="3">
-        <v>46237</v>
+        <v>46171</v>
       </c>
       <c r="J52" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K52" t="s">
         <v>5</v>
       </c>
       <c r="L52" s="3">
-        <v>46113</v>
+        <v>46133</v>
       </c>
       <c r="M52" t="s">
         <v>6</v>
@@ -3323,28 +3359,28 @@
         <v>0</v>
       </c>
       <c r="E53" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F53" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="G53" s="3">
-        <v>46113</v>
+        <v>46133</v>
       </c>
       <c r="H53" s="3">
-        <v>46224</v>
+        <v>46170</v>
       </c>
       <c r="I53" s="3">
-        <v>46227</v>
+        <v>46171</v>
       </c>
       <c r="J53" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K53" t="s">
         <v>5</v>
       </c>
       <c r="L53" s="3">
-        <v>46113</v>
+        <v>46133</v>
       </c>
       <c r="M53" t="s">
         <v>6</v>
@@ -3364,7 +3400,7 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C54" s="2">
         <v>1</v>
@@ -3373,19 +3409,19 @@
         <v>0</v>
       </c>
       <c r="E54" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F54" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G54" s="3">
-        <v>46114</v>
+        <v>46133</v>
       </c>
       <c r="H54" s="3">
-        <v>46149</v>
+        <v>46170</v>
       </c>
       <c r="I54" s="3">
-        <v>46153</v>
+        <v>46171</v>
       </c>
       <c r="J54" t="s">
         <v>4</v>
@@ -3394,7 +3430,7 @@
         <v>5</v>
       </c>
       <c r="L54" s="3">
-        <v>46114</v>
+        <v>46133</v>
       </c>
       <c r="M54" t="s">
         <v>6</v>
@@ -3414,7 +3450,7 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C55" s="2">
         <v>1</v>
@@ -3429,22 +3465,22 @@
         <v>117</v>
       </c>
       <c r="G55" s="3">
-        <v>46114</v>
+        <v>46136</v>
       </c>
       <c r="H55" s="3">
-        <v>46149</v>
+        <v>46136</v>
       </c>
       <c r="I55" s="3">
-        <v>46153</v>
+        <v>46141</v>
       </c>
       <c r="J55" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K55" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L55" s="3">
-        <v>46114</v>
+        <v>46136</v>
       </c>
       <c r="M55" t="s">
         <v>6</v>
@@ -3464,7 +3500,7 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C56" s="2">
         <v>1</v>
@@ -3473,28 +3509,28 @@
         <v>0</v>
       </c>
       <c r="E56" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="F56" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="G56" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="H56" s="3">
-        <v>46178</v>
+        <v>46136</v>
       </c>
       <c r="I56" s="3">
-        <v>46181</v>
+        <v>46141</v>
       </c>
       <c r="J56" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K56" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L56" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="M56" t="s">
         <v>6</v>
@@ -3514,7 +3550,7 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C57" s="2">
         <v>1</v>
@@ -3523,28 +3559,28 @@
         <v>0</v>
       </c>
       <c r="E57" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="F57" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="G57" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="H57" s="3">
-        <v>46174</v>
+        <v>46136</v>
       </c>
       <c r="I57" s="3">
-        <v>46177</v>
+        <v>46141</v>
       </c>
       <c r="J57" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K57" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L57" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="M57" t="s">
         <v>6</v>
@@ -3564,7 +3600,7 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C58" s="2">
         <v>1</v>
@@ -3573,28 +3609,28 @@
         <v>0</v>
       </c>
       <c r="E58" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="F58" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G58" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="H58" s="3">
-        <v>46170</v>
+        <v>46136</v>
       </c>
       <c r="I58" s="3">
-        <v>46171</v>
+        <v>46141</v>
       </c>
       <c r="J58" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K58" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L58" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="M58" t="s">
         <v>6</v>
@@ -3614,7 +3650,7 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C59" s="2">
         <v>1</v>
@@ -3629,22 +3665,22 @@
         <v>123</v>
       </c>
       <c r="G59" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="H59" s="3">
-        <v>46170</v>
+        <v>46136</v>
       </c>
       <c r="I59" s="3">
-        <v>46171</v>
+        <v>46141</v>
       </c>
       <c r="J59" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K59" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L59" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="M59" t="s">
         <v>6</v>
@@ -3664,37 +3700,37 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
+        <v>124</v>
+      </c>
+      <c r="C60" s="2">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
         <v>125</v>
       </c>
-      <c r="C60" s="2">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2">
-        <v>0</v>
-      </c>
-      <c r="E60" t="s">
-        <v>122</v>
-      </c>
       <c r="F60" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G60" s="3">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="H60" s="3">
         <v>46170</v>
       </c>
       <c r="I60" s="3">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="J60" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="K60" t="s">
         <v>5</v>
       </c>
       <c r="L60" s="3">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="M60" t="s">
         <v>6</v>
@@ -3714,7 +3750,7 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C61" s="2">
         <v>1</v>
@@ -3723,28 +3759,28 @@
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F61" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G61" s="3">
-        <v>46134</v>
+        <v>46139</v>
       </c>
       <c r="H61" s="3">
-        <v>46134</v>
+        <v>46164</v>
       </c>
       <c r="I61" s="3">
+        <v>46169</v>
+      </c>
+      <c r="J61" t="s">
+        <v>30</v>
+      </c>
+      <c r="K61" t="s">
+        <v>5</v>
+      </c>
+      <c r="L61" s="3">
         <v>46139</v>
-      </c>
-      <c r="J61" t="s">
-        <v>4</v>
-      </c>
-      <c r="K61" t="s">
-        <v>5</v>
-      </c>
-      <c r="L61" s="3">
-        <v>46134</v>
       </c>
       <c r="M61" t="s">
         <v>6</v>
@@ -3764,7 +3800,7 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C62" s="2">
         <v>1</v>
@@ -3773,28 +3809,28 @@
         <v>0</v>
       </c>
       <c r="E62" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F62" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G62" s="3">
-        <v>46134</v>
+        <v>46140</v>
       </c>
       <c r="H62" s="3">
-        <v>46135</v>
+        <v>46183</v>
       </c>
       <c r="I62" s="3">
+        <v>46190</v>
+      </c>
+      <c r="J62" t="s">
+        <v>54</v>
+      </c>
+      <c r="K62" t="s">
+        <v>5</v>
+      </c>
+      <c r="L62" s="3">
         <v>46140</v>
-      </c>
-      <c r="J62" t="s">
-        <v>4</v>
-      </c>
-      <c r="K62" t="s">
-        <v>5</v>
-      </c>
-      <c r="L62" s="3">
-        <v>46134</v>
       </c>
       <c r="M62" t="s">
         <v>6</v>
@@ -3814,37 +3850,37 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
+        <v>133</v>
+      </c>
+      <c r="C63" s="2">
+        <v>1</v>
+      </c>
+      <c r="D63" s="2">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>131</v>
+      </c>
+      <c r="F63" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="2">
-        <v>1</v>
-      </c>
-      <c r="D63" s="2">
-        <v>0</v>
-      </c>
-      <c r="E63" t="s">
-        <v>133</v>
-      </c>
-      <c r="F63" t="s">
-        <v>134</v>
-      </c>
       <c r="G63" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="H63" s="3">
-        <v>46139</v>
+        <v>46183</v>
       </c>
       <c r="I63" s="3">
-        <v>46142</v>
+        <v>46190</v>
       </c>
       <c r="J63" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="K63" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L63" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="M63" t="s">
         <v>6</v>
@@ -3864,37 +3900,37 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
+        <v>134</v>
+      </c>
+      <c r="C64" s="2">
+        <v>1</v>
+      </c>
+      <c r="D64" s="2">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
         <v>135</v>
       </c>
-      <c r="C64" s="2">
-        <v>1</v>
-      </c>
-      <c r="D64" s="2">
-        <v>0</v>
-      </c>
-      <c r="E64" t="s">
-        <v>133</v>
-      </c>
       <c r="F64" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G64" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="H64" s="3">
-        <v>46139</v>
+        <v>46176</v>
       </c>
       <c r="I64" s="3">
-        <v>46142</v>
+        <v>46182</v>
       </c>
       <c r="J64" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K64" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L64" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="M64" t="s">
         <v>6</v>
@@ -3914,37 +3950,37 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
+        <v>137</v>
+      </c>
+      <c r="C65" s="2">
+        <v>1</v>
+      </c>
+      <c r="D65" s="2">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>135</v>
+      </c>
+      <c r="F65" t="s">
         <v>136</v>
       </c>
-      <c r="C65" s="2">
-        <v>1</v>
-      </c>
-      <c r="D65" s="2">
-        <v>0</v>
-      </c>
-      <c r="E65" t="s">
-        <v>133</v>
-      </c>
-      <c r="F65" t="s">
-        <v>134</v>
-      </c>
       <c r="G65" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="H65" s="3">
-        <v>46139</v>
+        <v>46176</v>
       </c>
       <c r="I65" s="3">
-        <v>46142</v>
+        <v>46182</v>
       </c>
       <c r="J65" t="s">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="K65" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L65" s="3">
-        <v>46136</v>
+        <v>46140</v>
       </c>
       <c r="M65" t="s">
         <v>6</v>
@@ -3964,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C66" s="2">
         <v>1</v>
@@ -3973,28 +4009,28 @@
         <v>0</v>
       </c>
       <c r="E66" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F66" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="G66" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H66" s="3">
-        <v>46139</v>
+        <v>46150</v>
       </c>
       <c r="I66" s="3">
+        <v>46154</v>
+      </c>
+      <c r="J66" t="s">
+        <v>30</v>
+      </c>
+      <c r="K66" t="s">
+        <v>5</v>
+      </c>
+      <c r="L66" s="3">
         <v>46142</v>
-      </c>
-      <c r="J66" t="s">
-        <v>4</v>
-      </c>
-      <c r="K66" t="s">
-        <v>66</v>
-      </c>
-      <c r="L66" s="3">
-        <v>46136</v>
       </c>
       <c r="M66" t="s">
         <v>6</v>
@@ -4014,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C67" s="2">
         <v>1</v>
@@ -4029,22 +4065,22 @@
         <v>140</v>
       </c>
       <c r="G67" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H67" s="3">
-        <v>46136</v>
+        <v>46150</v>
       </c>
       <c r="I67" s="3">
-        <v>46141</v>
+        <v>46154</v>
       </c>
       <c r="J67" t="s">
         <v>4</v>
       </c>
       <c r="K67" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L67" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M67" t="s">
         <v>6</v>
@@ -4064,7 +4100,7 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C68" s="2">
         <v>1</v>
@@ -4079,22 +4115,22 @@
         <v>140</v>
       </c>
       <c r="G68" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H68" s="3">
-        <v>46136</v>
+        <v>46150</v>
       </c>
       <c r="I68" s="3">
-        <v>46141</v>
+        <v>46154</v>
       </c>
       <c r="J68" t="s">
         <v>4</v>
       </c>
       <c r="K68" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L68" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M68" t="s">
         <v>6</v>
@@ -4114,7 +4150,7 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C69" s="2">
         <v>1</v>
@@ -4129,22 +4165,22 @@
         <v>140</v>
       </c>
       <c r="G69" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H69" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I69" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J69" t="s">
         <v>4</v>
       </c>
       <c r="K69" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L69" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M69" t="s">
         <v>6</v>
@@ -4164,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C70" s="2">
         <v>1</v>
@@ -4179,22 +4215,22 @@
         <v>140</v>
       </c>
       <c r="G70" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H70" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I70" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J70" t="s">
         <v>4</v>
       </c>
       <c r="K70" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L70" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M70" t="s">
         <v>6</v>
@@ -4214,7 +4250,7 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C71" s="2">
         <v>1</v>
@@ -4223,28 +4259,28 @@
         <v>0</v>
       </c>
       <c r="E71" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="F71" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="G71" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H71" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I71" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J71" t="s">
         <v>4</v>
       </c>
       <c r="K71" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="L71" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M71" t="s">
         <v>6</v>
@@ -4264,7 +4300,7 @@
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C72" s="2">
         <v>1</v>
@@ -4273,28 +4309,28 @@
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="F72" t="s">
-        <v>147</v>
+        <v>97</v>
       </c>
       <c r="G72" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="H72" s="3">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="I72" s="3">
-        <v>46174</v>
+        <v>46149</v>
       </c>
       <c r="J72" t="s">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="K72" t="s">
         <v>5</v>
       </c>
       <c r="L72" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="M72" t="s">
         <v>6</v>
@@ -4314,7 +4350,7 @@
         <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C73" s="2">
         <v>1</v>
@@ -4323,28 +4359,28 @@
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>149</v>
+        <v>96</v>
       </c>
       <c r="F73" t="s">
-        <v>150</v>
+        <v>97</v>
       </c>
       <c r="G73" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="H73" s="3">
-        <v>46164</v>
+        <v>46142</v>
       </c>
       <c r="I73" s="3">
-        <v>46169</v>
+        <v>46149</v>
       </c>
       <c r="J73" t="s">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="K73" t="s">
         <v>5</v>
       </c>
       <c r="L73" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="M73" t="s">
         <v>6</v>
@@ -4364,7 +4400,7 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C74" s="2">
         <v>1</v>
@@ -4373,28 +4409,28 @@
         <v>0</v>
       </c>
       <c r="E74" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="F74" t="s">
-        <v>14</v>
+        <v>97</v>
       </c>
       <c r="G74" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="H74" s="3">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="I74" s="3">
+        <v>46149</v>
+      </c>
+      <c r="J74" t="s">
+        <v>54</v>
+      </c>
+      <c r="K74" t="s">
+        <v>5</v>
+      </c>
+      <c r="L74" s="3">
         <v>46142</v>
-      </c>
-      <c r="J74" t="s">
-        <v>11</v>
-      </c>
-      <c r="K74" t="s">
-        <v>5</v>
-      </c>
-      <c r="L74" s="3">
-        <v>46139</v>
       </c>
       <c r="M74" t="s">
         <v>6</v>
@@ -4414,7 +4450,7 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C75" s="2">
         <v>1</v>
@@ -4423,28 +4459,28 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>153</v>
+        <v>96</v>
       </c>
       <c r="F75" t="s">
-        <v>154</v>
+        <v>97</v>
       </c>
       <c r="G75" s="3">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="H75" s="3">
-        <v>46140</v>
+        <v>46177</v>
       </c>
       <c r="I75" s="3">
+        <v>46183</v>
+      </c>
+      <c r="J75" t="s">
+        <v>30</v>
+      </c>
+      <c r="K75" t="s">
+        <v>5</v>
+      </c>
+      <c r="L75" s="3">
         <v>46142</v>
-      </c>
-      <c r="J75" t="s">
-        <v>4</v>
-      </c>
-      <c r="K75" t="s">
-        <v>5</v>
-      </c>
-      <c r="L75" s="3">
-        <v>46140</v>
       </c>
       <c r="M75" t="s">
         <v>6</v>
@@ -4464,7 +4500,7 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C76" s="2">
         <v>1</v>
@@ -4473,28 +4509,28 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="F76" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="G76" s="3">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="H76" s="3">
-        <v>46140</v>
+        <v>46177</v>
       </c>
       <c r="I76" s="3">
-        <v>46146</v>
+        <v>46183</v>
       </c>
       <c r="J76" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K76" t="s">
         <v>5</v>
       </c>
       <c r="L76" s="3">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="M76" t="s">
         <v>6</v>
@@ -4514,7 +4550,7 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C77" s="2">
         <v>1</v>
@@ -4523,28 +4559,28 @@
         <v>0</v>
       </c>
       <c r="E77" t="s">
-        <v>157</v>
+        <v>96</v>
       </c>
       <c r="F77" t="s">
-        <v>158</v>
+        <v>97</v>
       </c>
       <c r="G77" s="3">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="H77" s="3">
+        <v>46177</v>
+      </c>
+      <c r="I77" s="3">
         <v>46183</v>
       </c>
-      <c r="I77" s="3">
-        <v>46190</v>
-      </c>
       <c r="J77" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="K77" t="s">
         <v>5</v>
       </c>
       <c r="L77" s="3">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="M77" t="s">
         <v>6</v>
@@ -4564,7 +4600,7 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C78" s="2">
         <v>1</v>
@@ -4573,28 +4609,28 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F78" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G78" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H78" s="3">
-        <v>46183</v>
+        <v>46204</v>
       </c>
       <c r="I78" s="3">
-        <v>46190</v>
+        <v>46206</v>
       </c>
       <c r="J78" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="K78" t="s">
         <v>5</v>
       </c>
       <c r="L78" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M78" t="s">
         <v>6</v>
@@ -4614,7 +4650,7 @@
         <v>0</v>
       </c>
       <c r="B79" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C79" s="2">
         <v>1</v>
@@ -4623,28 +4659,28 @@
         <v>0</v>
       </c>
       <c r="E79" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F79" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G79" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H79" s="3">
-        <v>46176</v>
+        <v>46163</v>
       </c>
       <c r="I79" s="3">
-        <v>46182</v>
+        <v>46170</v>
       </c>
       <c r="J79" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="K79" t="s">
         <v>5</v>
       </c>
       <c r="L79" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M79" t="s">
         <v>6</v>
@@ -4664,7 +4700,7 @@
         <v>0</v>
       </c>
       <c r="B80" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C80" s="2">
         <v>1</v>
@@ -4673,28 +4709,28 @@
         <v>0</v>
       </c>
       <c r="E80" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F80" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G80" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H80" s="3">
-        <v>46176</v>
+        <v>46157</v>
       </c>
       <c r="I80" s="3">
-        <v>46182</v>
+        <v>46162</v>
       </c>
       <c r="J80" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="K80" t="s">
         <v>5</v>
       </c>
       <c r="L80" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M80" t="s">
         <v>6</v>
@@ -4714,7 +4750,7 @@
         <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C81" s="2">
         <v>1</v>
@@ -4723,28 +4759,28 @@
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F81" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G81" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H81" s="3">
-        <v>46140</v>
+        <v>46224</v>
       </c>
       <c r="I81" s="3">
-        <v>46147</v>
+        <v>46262</v>
       </c>
       <c r="J81" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K81" t="s">
         <v>5</v>
       </c>
       <c r="L81" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M81" t="s">
         <v>6</v>
@@ -4761,10 +4797,10 @@
     </row>
     <row r="82" spans="1:16">
       <c r="A82" t="s">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C82" s="2">
         <v>1</v>
@@ -4773,28 +4809,28 @@
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F82" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G82" s="3">
-        <v>46043</v>
+        <v>46148</v>
       </c>
       <c r="H82" s="3">
-        <v>46051</v>
+        <v>46212</v>
       </c>
       <c r="I82" s="3">
-        <v>46057</v>
+        <v>46219</v>
       </c>
       <c r="J82" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="K82" t="s">
-        <v>171</v>
+        <v>5</v>
       </c>
       <c r="L82" s="3">
-        <v>46043</v>
+        <v>46148</v>
       </c>
       <c r="M82" t="s">
         <v>6</v>
@@ -4811,51 +4847,301 @@
     </row>
     <row r="83" spans="1:16">
       <c r="A83" t="s">
+        <v>0</v>
+      </c>
+      <c r="B83" t="s">
         <v>167</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" s="2">
+        <v>1</v>
+      </c>
+      <c r="D83" s="2">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>168</v>
+      </c>
+      <c r="F83" t="s">
+        <v>169</v>
+      </c>
+      <c r="G83" s="3">
+        <v>46148</v>
+      </c>
+      <c r="H83" s="3">
+        <v>46197</v>
+      </c>
+      <c r="I83" s="3">
+        <v>46202</v>
+      </c>
+      <c r="J83" t="s">
+        <v>30</v>
+      </c>
+      <c r="K83" t="s">
+        <v>5</v>
+      </c>
+      <c r="L83" s="3">
+        <v>46148</v>
+      </c>
+      <c r="M83" t="s">
+        <v>6</v>
+      </c>
+      <c r="N83" t="s">
+        <v>7</v>
+      </c>
+      <c r="O83" t="s">
+        <v>8</v>
+      </c>
+      <c r="P83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" t="s">
+        <v>170</v>
+      </c>
+      <c r="C84" s="2">
+        <v>1</v>
+      </c>
+      <c r="D84" s="2">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>171</v>
+      </c>
+      <c r="F84" t="s">
         <v>172</v>
       </c>
-      <c r="C83" s="2">
-        <v>1</v>
-      </c>
-      <c r="D83" s="2">
-        <v>0</v>
-      </c>
-      <c r="E83" t="s">
+      <c r="G84" s="3">
+        <v>46148</v>
+      </c>
+      <c r="H84" s="3">
+        <v>46191</v>
+      </c>
+      <c r="I84" s="3">
+        <v>46197</v>
+      </c>
+      <c r="J84" t="s">
+        <v>30</v>
+      </c>
+      <c r="K84" t="s">
+        <v>5</v>
+      </c>
+      <c r="L84" s="3">
+        <v>46148</v>
+      </c>
+      <c r="M84" t="s">
+        <v>6</v>
+      </c>
+      <c r="N84" t="s">
+        <v>7</v>
+      </c>
+      <c r="O84" t="s">
+        <v>8</v>
+      </c>
+      <c r="P84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
         <v>173</v>
       </c>
-      <c r="F83" t="s">
+      <c r="C85" s="2">
+        <v>1</v>
+      </c>
+      <c r="D85" s="2">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
         <v>174</v>
       </c>
-      <c r="G83" s="3">
-        <v>46140</v>
-      </c>
-      <c r="H83" s="3">
-        <v>46140</v>
-      </c>
-      <c r="I83" s="3">
-        <v>46147</v>
-      </c>
-      <c r="J83" t="s">
-        <v>11</v>
-      </c>
-      <c r="K83" t="s">
-        <v>171</v>
-      </c>
-      <c r="L83" s="3">
-        <v>46140</v>
-      </c>
-      <c r="M83" t="s">
-        <v>6</v>
-      </c>
-      <c r="N83" t="s">
-        <v>7</v>
-      </c>
-      <c r="O83" t="s">
-        <v>8</v>
-      </c>
-      <c r="P83" t="s">
+      <c r="F85" t="s">
+        <v>175</v>
+      </c>
+      <c r="G85" s="3">
+        <v>46148</v>
+      </c>
+      <c r="H85" s="3">
+        <v>46204</v>
+      </c>
+      <c r="I85" s="3">
+        <v>46204</v>
+      </c>
+      <c r="J85" t="s">
+        <v>30</v>
+      </c>
+      <c r="K85" t="s">
+        <v>5</v>
+      </c>
+      <c r="L85" s="3">
+        <v>46148</v>
+      </c>
+      <c r="M85" t="s">
+        <v>6</v>
+      </c>
+      <c r="N85" t="s">
+        <v>7</v>
+      </c>
+      <c r="O85" t="s">
+        <v>8</v>
+      </c>
+      <c r="P85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16">
+      <c r="A86" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" t="s">
+        <v>176</v>
+      </c>
+      <c r="C86" s="2">
+        <v>1</v>
+      </c>
+      <c r="D86" s="2">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>177</v>
+      </c>
+      <c r="F86" t="s">
+        <v>178</v>
+      </c>
+      <c r="G86" s="3">
+        <v>46148</v>
+      </c>
+      <c r="H86" s="3">
+        <v>46199</v>
+      </c>
+      <c r="I86" s="3">
+        <v>46204</v>
+      </c>
+      <c r="J86" t="s">
+        <v>30</v>
+      </c>
+      <c r="K86" t="s">
+        <v>5</v>
+      </c>
+      <c r="L86" s="3">
+        <v>46148</v>
+      </c>
+      <c r="M86" t="s">
+        <v>6</v>
+      </c>
+      <c r="N86" t="s">
+        <v>7</v>
+      </c>
+      <c r="O86" t="s">
+        <v>8</v>
+      </c>
+      <c r="P86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16">
+      <c r="A87" t="s">
+        <v>0</v>
+      </c>
+      <c r="B87" t="s">
+        <v>179</v>
+      </c>
+      <c r="C87" s="2">
+        <v>1</v>
+      </c>
+      <c r="D87" s="2">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>180</v>
+      </c>
+      <c r="F87" t="s">
+        <v>181</v>
+      </c>
+      <c r="G87" s="3">
+        <v>46148</v>
+      </c>
+      <c r="H87" s="3">
+        <v>46279</v>
+      </c>
+      <c r="I87" s="3">
+        <v>46281</v>
+      </c>
+      <c r="J87" t="s">
+        <v>30</v>
+      </c>
+      <c r="K87" t="s">
+        <v>5</v>
+      </c>
+      <c r="L87" s="3">
+        <v>46148</v>
+      </c>
+      <c r="M87" t="s">
+        <v>6</v>
+      </c>
+      <c r="N87" t="s">
+        <v>7</v>
+      </c>
+      <c r="O87" t="s">
+        <v>8</v>
+      </c>
+      <c r="P87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16">
+      <c r="A88" t="s">
+        <v>182</v>
+      </c>
+      <c r="B88" t="s">
+        <v>183</v>
+      </c>
+      <c r="C88" s="2">
+        <v>1</v>
+      </c>
+      <c r="D88" s="2">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>184</v>
+      </c>
+      <c r="F88" t="s">
+        <v>185</v>
+      </c>
+      <c r="G88" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H88" s="3">
+        <v>46051</v>
+      </c>
+      <c r="I88" s="3">
+        <v>46057</v>
+      </c>
+      <c r="J88" t="s">
+        <v>4</v>
+      </c>
+      <c r="K88" t="s">
+        <v>186</v>
+      </c>
+      <c r="L88" s="3">
+        <v>46043</v>
+      </c>
+      <c r="M88" t="s">
+        <v>6</v>
+      </c>
+      <c r="N88" t="s">
+        <v>7</v>
+      </c>
+      <c r="O88" t="s">
+        <v>8</v>
+      </c>
+      <c r="P88" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard and system updates
</commit_message>
<xml_diff>
--- a/Newdata/半品未撥.XLSX
+++ b/Newdata/半品未撥.XLSX
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="200">
   <si>
     <t>ZP02</t>
   </si>
@@ -130,6 +130,9 @@
     <t>自動頭HF-AU,031911_1°-BBT50-45°-4K-C-F</t>
   </si>
   <si>
+    <t>REL  PCNF PRC  MANC SETC</t>
+  </si>
+  <si>
     <t>200006568</t>
   </si>
   <si>
@@ -139,15 +142,6 @@
     <t>自動頭HF-AU,031911_2.5°-BBT50-45°-4K-C-F</t>
   </si>
   <si>
-    <t>200006575</t>
-  </si>
-  <si>
-    <t>080300017908</t>
-  </si>
-  <si>
-    <t>自動頭HF-A90,031944_1°-BT50-45°-4K-0</t>
-  </si>
-  <si>
     <t>200006576</t>
   </si>
   <si>
@@ -325,39 +319,12 @@
     <t>080100113504</t>
   </si>
   <si>
-    <t>200006659</t>
-  </si>
-  <si>
-    <t>080200530500</t>
-  </si>
-  <si>
-    <t>MVP-8機頭D15K,021581_#40,38F18,C</t>
-  </si>
-  <si>
-    <t>200006660</t>
-  </si>
-  <si>
     <t>200006681</t>
   </si>
   <si>
     <t>200006682</t>
   </si>
   <si>
-    <t>200006683</t>
-  </si>
-  <si>
-    <t>080200070801</t>
-  </si>
-  <si>
-    <t>L800機頭P12K,021615_BBT40,5GT,0AW45</t>
-  </si>
-  <si>
-    <t>200006684</t>
-  </si>
-  <si>
-    <t>200006685</t>
-  </si>
-  <si>
     <t>200006693</t>
   </si>
   <si>
@@ -394,40 +361,7 @@
     <t>MVP-16機頭D20K,021825_A63,38F18,C</t>
   </si>
   <si>
-    <t>200006699</t>
-  </si>
-  <si>
-    <t>080100050303</t>
-  </si>
-  <si>
-    <t>D20K 主軸,010683_A63,M50,CW</t>
-  </si>
-  <si>
-    <t>200006703</t>
-  </si>
-  <si>
-    <t>080200422904</t>
-  </si>
-  <si>
-    <t>HEP機頭G8K,011194_780,55A18,C</t>
-  </si>
-  <si>
-    <t>200006704</t>
-  </si>
-  <si>
-    <t>200006705</t>
-  </si>
-  <si>
-    <t>080100037203</t>
-  </si>
-  <si>
-    <t>D8K 主軸,021274_BT50,M50,C045</t>
-  </si>
-  <si>
-    <t>200006706</t>
-  </si>
-  <si>
-    <t>200006708</t>
+    <t>200006711</t>
   </si>
   <si>
     <t>080200546502</t>
@@ -436,39 +370,12 @@
     <t>MVP11機頭D15K,031859_#40,32F18,0</t>
   </si>
   <si>
-    <t>200006709</t>
-  </si>
-  <si>
-    <t>200006710</t>
-  </si>
-  <si>
-    <t>200006711</t>
-  </si>
-  <si>
     <t>200006712</t>
   </si>
   <si>
     <t>200006713</t>
   </si>
   <si>
-    <t>200006714</t>
-  </si>
-  <si>
-    <t>200006715</t>
-  </si>
-  <si>
-    <t>200006716</t>
-  </si>
-  <si>
-    <t>200006717</t>
-  </si>
-  <si>
-    <t>200006718</t>
-  </si>
-  <si>
-    <t>200006719</t>
-  </si>
-  <si>
     <t>200006720</t>
   </si>
   <si>
@@ -487,15 +394,6 @@
     <t>HSA機頭G8K,011147_1000,55A22,C</t>
   </si>
   <si>
-    <t>200006722</t>
-  </si>
-  <si>
-    <t>080100048401</t>
-  </si>
-  <si>
-    <t>G8K 主軸,011119_BBT50,M50,C045</t>
-  </si>
-  <si>
     <t>200006723</t>
   </si>
   <si>
@@ -557,6 +455,99 @@
   </si>
   <si>
     <t>L2100機頭D12K,021634_#40,48F23</t>
+  </si>
+  <si>
+    <t>200006731</t>
+  </si>
+  <si>
+    <t>080100145601</t>
+  </si>
+  <si>
+    <t>D6K 主軸,010801_BT50,M50E,0045</t>
+  </si>
+  <si>
+    <t>200006732</t>
+  </si>
+  <si>
+    <t>080300016308</t>
+  </si>
+  <si>
+    <t>自動頭HF-A90,031944_2.5°-BT50-45°-4K-0</t>
+  </si>
+  <si>
+    <t>200006734</t>
+  </si>
+  <si>
+    <t>080100022704</t>
+  </si>
+  <si>
+    <t>G6K 主軸,021327_BT50,0045</t>
+  </si>
+  <si>
+    <t>200006735</t>
+  </si>
+  <si>
+    <t>080200014502</t>
+  </si>
+  <si>
+    <t>EA機頭G6K,011166_Z1000,60A30,C</t>
+  </si>
+  <si>
+    <t>200006736</t>
+  </si>
+  <si>
+    <t>080100015101</t>
+  </si>
+  <si>
+    <t>D6K 主軸,010801_BT50,M50E,C045</t>
+  </si>
+  <si>
+    <t>200006737</t>
+  </si>
+  <si>
+    <t>080300020609</t>
+  </si>
+  <si>
+    <t>自動頭HF-AU,031911_1°-BT50-45°-4K-C-F</t>
+  </si>
+  <si>
+    <t>200006738</t>
+  </si>
+  <si>
+    <t>080200548000</t>
+  </si>
+  <si>
+    <t>MVP13機頭D15K,011237_#40,38F18</t>
+  </si>
+  <si>
+    <t>200006739</t>
+  </si>
+  <si>
+    <t>200006740</t>
+  </si>
+  <si>
+    <t>200006741</t>
+  </si>
+  <si>
+    <t>200006742</t>
+  </si>
+  <si>
+    <t>080200243400</t>
+  </si>
+  <si>
+    <t>MVP11機頭P12K,021415_BBT40,5GT,0AW45</t>
+  </si>
+  <si>
+    <t>REL  PRC  LKD  MACM SETC</t>
+  </si>
+  <si>
+    <t>200006743</t>
+  </si>
+  <si>
+    <t>080100036004</t>
+  </si>
+  <si>
+    <t>G6K 主軸,021327_BBT50,C045</t>
   </si>
   <si>
     <t>ZP09</t>
@@ -724,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P88"/>
+  <dimension ref="A1:P79"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="6" customWidth="1"/>
@@ -747,52 +738,52 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -1724,7 +1715,7 @@
         <v>46171</v>
       </c>
       <c r="J20" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="K20" t="s">
         <v>5</v>
@@ -1750,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C21" s="2">
         <v>1</v>
@@ -1759,10 +1750,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G21" s="3">
         <v>46083</v>
@@ -1800,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -1809,22 +1800,22 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G22" s="3">
         <v>46086</v>
       </c>
       <c r="H22" s="3">
-        <v>46167</v>
+        <v>46213</v>
       </c>
       <c r="I22" s="3">
-        <v>46185</v>
+        <v>46217</v>
       </c>
       <c r="J22" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K22" t="s">
         <v>5</v>
@@ -1850,7 +1841,7 @@
         <v>0</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C23" s="2">
         <v>1</v>
@@ -1859,19 +1850,19 @@
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G23" s="3">
         <v>46086</v>
       </c>
       <c r="H23" s="3">
-        <v>46213</v>
+        <v>46191</v>
       </c>
       <c r="I23" s="3">
-        <v>46217</v>
+        <v>46210</v>
       </c>
       <c r="J23" t="s">
         <v>30</v>
@@ -1900,7 +1891,7 @@
         <v>0</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C24" s="2">
         <v>1</v>
@@ -1909,28 +1900,28 @@
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G24" s="3">
-        <v>46086</v>
+        <v>46090</v>
       </c>
       <c r="H24" s="3">
-        <v>46191</v>
+        <v>46170</v>
       </c>
       <c r="I24" s="3">
-        <v>46210</v>
+        <v>46175</v>
       </c>
       <c r="J24" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="K24" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L24" s="3">
-        <v>46086</v>
+        <v>46090</v>
       </c>
       <c r="M24" t="s">
         <v>6</v>
@@ -1950,7 +1941,7 @@
         <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -1959,25 +1950,25 @@
         <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F25" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G25" s="3">
         <v>46090</v>
       </c>
       <c r="H25" s="3">
-        <v>46170</v>
+        <v>46206</v>
       </c>
       <c r="I25" s="3">
-        <v>46175</v>
+        <v>46210</v>
       </c>
       <c r="J25" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="K25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L25" s="3">
         <v>46090</v>
@@ -2000,7 +1991,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -2009,25 +2000,25 @@
         <v>0</v>
       </c>
       <c r="E26" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G26" s="3">
         <v>46090</v>
       </c>
       <c r="H26" s="3">
-        <v>46206</v>
+        <v>46202</v>
       </c>
       <c r="I26" s="3">
-        <v>46210</v>
+        <v>46205</v>
       </c>
       <c r="J26" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L26" s="3">
         <v>46090</v>
@@ -2050,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
@@ -2059,28 +2050,28 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G27" s="3">
-        <v>46090</v>
+        <v>46092</v>
       </c>
       <c r="H27" s="3">
-        <v>46202</v>
+        <v>46092</v>
       </c>
       <c r="I27" s="3">
-        <v>46205</v>
+        <v>46094</v>
       </c>
       <c r="J27" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K27" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L27" s="3">
-        <v>46090</v>
+        <v>46092</v>
       </c>
       <c r="M27" t="s">
         <v>6</v>
@@ -2100,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
@@ -2109,28 +2100,28 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F28" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G28" s="3">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="H28" s="3">
-        <v>46092</v>
+        <v>46167</v>
       </c>
       <c r="I28" s="3">
-        <v>46094</v>
+        <v>46169</v>
       </c>
       <c r="J28" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K28" t="s">
         <v>5</v>
       </c>
       <c r="L28" s="3">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="M28" t="s">
         <v>6</v>
@@ -2150,19 +2141,19 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="2">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F29" t="s">
         <v>65</v>
-      </c>
-      <c r="C29" s="2">
-        <v>1</v>
-      </c>
-      <c r="D29" s="2">
-        <v>0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>66</v>
-      </c>
-      <c r="F29" t="s">
-        <v>67</v>
       </c>
       <c r="G29" s="3">
         <v>46093</v>
@@ -2200,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C30" s="2">
         <v>1</v>
@@ -2209,10 +2200,10 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G30" s="3">
         <v>46093</v>
@@ -2224,7 +2215,7 @@
         <v>46169</v>
       </c>
       <c r="J30" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="K30" t="s">
         <v>5</v>
@@ -2259,28 +2250,28 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="F31" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G31" s="3">
-        <v>46093</v>
+        <v>46105</v>
       </c>
       <c r="H31" s="3">
-        <v>46167</v>
+        <v>46219</v>
       </c>
       <c r="I31" s="3">
-        <v>46169</v>
+        <v>46223</v>
       </c>
       <c r="J31" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="K31" t="s">
         <v>5</v>
       </c>
       <c r="L31" s="3">
-        <v>46093</v>
+        <v>46105</v>
       </c>
       <c r="M31" t="s">
         <v>6</v>
@@ -2300,31 +2291,31 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="2">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
         <v>71</v>
       </c>
-      <c r="C32" s="2">
-        <v>1</v>
-      </c>
-      <c r="D32" s="2">
-        <v>0</v>
-      </c>
-      <c r="E32" t="s">
-        <v>57</v>
-      </c>
       <c r="F32" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G32" s="3">
         <v>46105</v>
       </c>
       <c r="H32" s="3">
-        <v>46219</v>
+        <v>46212</v>
       </c>
       <c r="I32" s="3">
-        <v>46223</v>
+        <v>46218</v>
       </c>
       <c r="J32" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K32" t="s">
         <v>5</v>
@@ -2350,7 +2341,7 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -2359,28 +2350,28 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F33" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G33" s="3">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="H33" s="3">
-        <v>46212</v>
+        <v>46227</v>
       </c>
       <c r="I33" s="3">
-        <v>46218</v>
+        <v>46231</v>
       </c>
       <c r="J33" t="s">
         <v>4</v>
       </c>
       <c r="K33" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L33" s="3">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="M33" t="s">
         <v>6</v>
@@ -2400,7 +2391,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C34" s="2">
         <v>1</v>
@@ -2409,25 +2400,25 @@
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G34" s="3">
         <v>46106</v>
       </c>
       <c r="H34" s="3">
-        <v>46227</v>
+        <v>46211</v>
       </c>
       <c r="I34" s="3">
-        <v>46231</v>
+        <v>46216</v>
       </c>
       <c r="J34" t="s">
         <v>4</v>
       </c>
       <c r="K34" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L34" s="3">
         <v>46106</v>
@@ -2450,7 +2441,7 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C35" s="2">
         <v>1</v>
@@ -2459,25 +2450,25 @@
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G35" s="3">
         <v>46106</v>
       </c>
       <c r="H35" s="3">
-        <v>46211</v>
+        <v>46205</v>
       </c>
       <c r="I35" s="3">
-        <v>46216</v>
+        <v>46210</v>
       </c>
       <c r="J35" t="s">
         <v>4</v>
       </c>
       <c r="K35" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L35" s="3">
         <v>46106</v>
@@ -2500,7 +2491,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
@@ -2509,25 +2500,25 @@
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G36" s="3">
         <v>46106</v>
       </c>
       <c r="H36" s="3">
-        <v>46205</v>
+        <v>46225</v>
       </c>
       <c r="I36" s="3">
-        <v>46210</v>
+        <v>46226</v>
       </c>
       <c r="J36" t="s">
         <v>4</v>
       </c>
       <c r="K36" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L36" s="3">
         <v>46106</v>
@@ -2550,7 +2541,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C37" s="2">
         <v>1</v>
@@ -2559,25 +2550,25 @@
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="F37" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="G37" s="3">
         <v>46106</v>
       </c>
       <c r="H37" s="3">
-        <v>46225</v>
+        <v>46219</v>
       </c>
       <c r="I37" s="3">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="J37" t="s">
         <v>4</v>
       </c>
       <c r="K37" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L37" s="3">
         <v>46106</v>
@@ -2600,37 +2591,37 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
         <v>87</v>
       </c>
-      <c r="C38" s="2">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2">
-        <v>0</v>
-      </c>
-      <c r="E38" t="s">
-        <v>60</v>
-      </c>
       <c r="F38" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="G38" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="H38" s="3">
-        <v>46219</v>
+        <v>46168</v>
       </c>
       <c r="I38" s="3">
-        <v>46224</v>
+        <v>46170</v>
       </c>
       <c r="J38" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K38" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L38" s="3">
-        <v>46106</v>
+        <v>46113</v>
       </c>
       <c r="M38" t="s">
         <v>6</v>
@@ -2650,19 +2641,19 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
+        <v>89</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>87</v>
+      </c>
+      <c r="F39" t="s">
         <v>88</v>
-      </c>
-      <c r="C39" s="2">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2">
-        <v>0</v>
-      </c>
-      <c r="E39" t="s">
-        <v>89</v>
-      </c>
-      <c r="F39" t="s">
-        <v>90</v>
       </c>
       <c r="G39" s="3">
         <v>46113</v>
@@ -2700,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" s="2">
         <v>1</v>
@@ -2709,10 +2700,10 @@
         <v>0</v>
       </c>
       <c r="E40" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F40" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G40" s="3">
         <v>46113</v>
@@ -2750,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C41" s="2">
         <v>1</v>
@@ -2759,19 +2750,19 @@
         <v>0</v>
       </c>
       <c r="E41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F41" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G41" s="3">
         <v>46113</v>
       </c>
       <c r="H41" s="3">
-        <v>46168</v>
+        <v>46232</v>
       </c>
       <c r="I41" s="3">
-        <v>46170</v>
+        <v>46234</v>
       </c>
       <c r="J41" t="s">
         <v>30</v>
@@ -2800,7 +2791,7 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C42" s="2">
         <v>1</v>
@@ -2809,10 +2800,10 @@
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F42" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G42" s="3">
         <v>46113</v>
@@ -2850,28 +2841,28 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
+        <v>93</v>
+      </c>
+      <c r="C43" s="2">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
         <v>94</v>
       </c>
-      <c r="C43" s="2">
-        <v>1</v>
-      </c>
-      <c r="D43" s="2">
-        <v>0</v>
-      </c>
-      <c r="E43" t="s">
-        <v>89</v>
-      </c>
       <c r="F43" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G43" s="3">
         <v>46113</v>
       </c>
       <c r="H43" s="3">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="I43" s="3">
-        <v>46234</v>
+        <v>46231</v>
       </c>
       <c r="J43" t="s">
         <v>30</v>
@@ -2900,19 +2891,19 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
+        <v>96</v>
+      </c>
+      <c r="C44" s="2">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2">
+        <v>0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>94</v>
+      </c>
+      <c r="F44" t="s">
         <v>95</v>
-      </c>
-      <c r="C44" s="2">
-        <v>1</v>
-      </c>
-      <c r="D44" s="2">
-        <v>0</v>
-      </c>
-      <c r="E44" t="s">
-        <v>96</v>
-      </c>
-      <c r="F44" t="s">
-        <v>97</v>
       </c>
       <c r="G44" s="3">
         <v>46113</v>
@@ -2950,28 +2941,28 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
+        <v>97</v>
+      </c>
+      <c r="C45" s="2">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="2">
-        <v>1</v>
-      </c>
-      <c r="D45" s="2">
-        <v>0</v>
-      </c>
-      <c r="E45" t="s">
-        <v>96</v>
-      </c>
       <c r="F45" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G45" s="3">
         <v>46113</v>
       </c>
       <c r="H45" s="3">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="I45" s="3">
-        <v>46231</v>
+        <v>46237</v>
       </c>
       <c r="J45" t="s">
         <v>30</v>
@@ -3000,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C46" s="2">
         <v>1</v>
@@ -3009,19 +3000,19 @@
         <v>0</v>
       </c>
       <c r="E46" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F46" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="G46" s="3">
         <v>46113</v>
       </c>
       <c r="H46" s="3">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="I46" s="3">
-        <v>46237</v>
+        <v>46227</v>
       </c>
       <c r="J46" t="s">
         <v>30</v>
@@ -3059,28 +3050,28 @@
         <v>0</v>
       </c>
       <c r="E47" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="F47" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G47" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="H47" s="3">
-        <v>46224</v>
+        <v>46178</v>
       </c>
       <c r="I47" s="3">
-        <v>46227</v>
+        <v>46181</v>
       </c>
       <c r="J47" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K47" t="s">
         <v>5</v>
       </c>
       <c r="L47" s="3">
-        <v>46113</v>
+        <v>46132</v>
       </c>
       <c r="M47" t="s">
         <v>6</v>
@@ -3100,7 +3091,7 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C48" s="2">
         <v>1</v>
@@ -3109,28 +3100,28 @@
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="F48" t="s">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="G48" s="3">
-        <v>46114</v>
+        <v>46132</v>
       </c>
       <c r="H48" s="3">
-        <v>46149</v>
+        <v>46174</v>
       </c>
       <c r="I48" s="3">
-        <v>46153</v>
+        <v>46177</v>
       </c>
       <c r="J48" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K48" t="s">
         <v>5</v>
       </c>
       <c r="L48" s="3">
-        <v>46114</v>
+        <v>46132</v>
       </c>
       <c r="M48" t="s">
         <v>6</v>
@@ -3150,7 +3141,7 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C49" s="2">
         <v>1</v>
@@ -3165,22 +3156,22 @@
         <v>106</v>
       </c>
       <c r="G49" s="3">
-        <v>46114</v>
+        <v>46136</v>
       </c>
       <c r="H49" s="3">
-        <v>46149</v>
+        <v>46136</v>
       </c>
       <c r="I49" s="3">
-        <v>46153</v>
+        <v>46141</v>
       </c>
       <c r="J49" t="s">
         <v>30</v>
       </c>
       <c r="K49" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L49" s="3">
-        <v>46114</v>
+        <v>46136</v>
       </c>
       <c r="M49" t="s">
         <v>6</v>
@@ -3200,7 +3191,7 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C50" s="2">
         <v>1</v>
@@ -3209,28 +3200,28 @@
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="F50" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="G50" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="H50" s="3">
-        <v>46178</v>
+        <v>46136</v>
       </c>
       <c r="I50" s="3">
-        <v>46181</v>
+        <v>46141</v>
       </c>
       <c r="J50" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K50" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L50" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="M50" t="s">
         <v>6</v>
@@ -3250,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C51" s="2">
         <v>1</v>
@@ -3259,28 +3250,28 @@
         <v>0</v>
       </c>
       <c r="E51" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="F51" t="s">
-        <v>29</v>
+        <v>106</v>
       </c>
       <c r="G51" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="H51" s="3">
-        <v>46174</v>
+        <v>46136</v>
       </c>
       <c r="I51" s="3">
-        <v>46177</v>
+        <v>46141</v>
       </c>
       <c r="J51" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K51" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L51" s="3">
-        <v>46132</v>
+        <v>46136</v>
       </c>
       <c r="M51" t="s">
         <v>6</v>
@@ -3300,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="B52" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C52" s="2">
         <v>1</v>
@@ -3309,28 +3300,28 @@
         <v>0</v>
       </c>
       <c r="E52" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="F52" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="G52" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="H52" s="3">
-        <v>46170</v>
+        <v>46136</v>
       </c>
       <c r="I52" s="3">
-        <v>46171</v>
+        <v>46141</v>
       </c>
       <c r="J52" t="s">
         <v>30</v>
       </c>
       <c r="K52" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L52" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="M52" t="s">
         <v>6</v>
@@ -3350,7 +3341,7 @@
         <v>0</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C53" s="2">
         <v>1</v>
@@ -3365,22 +3356,22 @@
         <v>112</v>
       </c>
       <c r="G53" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="H53" s="3">
-        <v>46170</v>
+        <v>46136</v>
       </c>
       <c r="I53" s="3">
-        <v>46171</v>
+        <v>46141</v>
       </c>
       <c r="J53" t="s">
         <v>30</v>
       </c>
       <c r="K53" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="L53" s="3">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="M53" t="s">
         <v>6</v>
@@ -3400,37 +3391,37 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
+        <v>113</v>
+      </c>
+      <c r="C54" s="2">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
         <v>114</v>
       </c>
-      <c r="C54" s="2">
-        <v>1</v>
-      </c>
-      <c r="D54" s="2">
-        <v>0</v>
-      </c>
-      <c r="E54" t="s">
-        <v>111</v>
-      </c>
       <c r="F54" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G54" s="3">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="H54" s="3">
         <v>46170</v>
       </c>
       <c r="I54" s="3">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="J54" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="K54" t="s">
         <v>5</v>
       </c>
       <c r="L54" s="3">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="M54" t="s">
         <v>6</v>
@@ -3450,7 +3441,7 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C55" s="2">
         <v>1</v>
@@ -3459,28 +3450,28 @@
         <v>0</v>
       </c>
       <c r="E55" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F55" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G55" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H55" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I55" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J55" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K55" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L55" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M55" t="s">
         <v>6</v>
@@ -3500,37 +3491,37 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
+        <v>119</v>
+      </c>
+      <c r="C56" s="2">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>117</v>
+      </c>
+      <c r="F56" t="s">
         <v>118</v>
       </c>
-      <c r="C56" s="2">
-        <v>1</v>
-      </c>
-      <c r="D56" s="2">
-        <v>0</v>
-      </c>
-      <c r="E56" t="s">
-        <v>116</v>
-      </c>
-      <c r="F56" t="s">
-        <v>117</v>
-      </c>
       <c r="G56" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H56" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I56" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J56" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K56" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L56" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M56" t="s">
         <v>6</v>
@@ -3550,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C57" s="2">
         <v>1</v>
@@ -3559,28 +3550,28 @@
         <v>0</v>
       </c>
       <c r="E57" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G57" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="H57" s="3">
-        <v>46136</v>
+        <v>46184</v>
       </c>
       <c r="I57" s="3">
-        <v>46141</v>
+        <v>46188</v>
       </c>
       <c r="J57" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K57" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L57" s="3">
-        <v>46136</v>
+        <v>46142</v>
       </c>
       <c r="M57" t="s">
         <v>6</v>
@@ -3600,7 +3591,7 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C58" s="2">
         <v>1</v>
@@ -3609,28 +3600,28 @@
         <v>0</v>
       </c>
       <c r="E58" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F58" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="G58" s="3">
-        <v>46136</v>
+        <v>46148</v>
       </c>
       <c r="H58" s="3">
-        <v>46136</v>
+        <v>46204</v>
       </c>
       <c r="I58" s="3">
-        <v>46141</v>
+        <v>46206</v>
       </c>
       <c r="J58" t="s">
         <v>30</v>
       </c>
       <c r="K58" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L58" s="3">
-        <v>46136</v>
+        <v>46148</v>
       </c>
       <c r="M58" t="s">
         <v>6</v>
@@ -3650,7 +3641,7 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C59" s="2">
         <v>1</v>
@@ -3659,28 +3650,28 @@
         <v>0</v>
       </c>
       <c r="E59" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F59" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G59" s="3">
-        <v>46136</v>
+        <v>46148</v>
       </c>
       <c r="H59" s="3">
-        <v>46136</v>
+        <v>46163</v>
       </c>
       <c r="I59" s="3">
-        <v>46141</v>
+        <v>46170</v>
       </c>
       <c r="J59" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="K59" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="L59" s="3">
-        <v>46136</v>
+        <v>46148</v>
       </c>
       <c r="M59" t="s">
         <v>6</v>
@@ -3700,7 +3691,7 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C60" s="2">
         <v>1</v>
@@ -3709,28 +3700,28 @@
         <v>0</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F60" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G60" s="3">
-        <v>46139</v>
+        <v>46148</v>
       </c>
       <c r="H60" s="3">
-        <v>46170</v>
+        <v>46185</v>
       </c>
       <c r="I60" s="3">
-        <v>46174</v>
+        <v>46226</v>
       </c>
       <c r="J60" t="s">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="K60" t="s">
         <v>5</v>
       </c>
       <c r="L60" s="3">
-        <v>46139</v>
+        <v>46148</v>
       </c>
       <c r="M60" t="s">
         <v>6</v>
@@ -3750,7 +3741,7 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C61" s="2">
         <v>1</v>
@@ -3759,28 +3750,28 @@
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F61" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G61" s="3">
-        <v>46139</v>
+        <v>46148</v>
       </c>
       <c r="H61" s="3">
-        <v>46164</v>
+        <v>46182</v>
       </c>
       <c r="I61" s="3">
-        <v>46169</v>
+        <v>46189</v>
       </c>
       <c r="J61" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K61" t="s">
         <v>5</v>
       </c>
       <c r="L61" s="3">
-        <v>46139</v>
+        <v>46148</v>
       </c>
       <c r="M61" t="s">
         <v>6</v>
@@ -3800,7 +3791,7 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C62" s="2">
         <v>1</v>
@@ -3809,28 +3800,28 @@
         <v>0</v>
       </c>
       <c r="E62" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F62" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="G62" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H62" s="3">
-        <v>46183</v>
+        <v>46197</v>
       </c>
       <c r="I62" s="3">
-        <v>46190</v>
+        <v>46202</v>
       </c>
       <c r="J62" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="K62" t="s">
         <v>5</v>
       </c>
       <c r="L62" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M62" t="s">
         <v>6</v>
@@ -3850,7 +3841,7 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C63" s="2">
         <v>1</v>
@@ -3859,28 +3850,28 @@
         <v>0</v>
       </c>
       <c r="E63" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F63" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="G63" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H63" s="3">
-        <v>46183</v>
+        <v>46191</v>
       </c>
       <c r="I63" s="3">
-        <v>46190</v>
+        <v>46197</v>
       </c>
       <c r="J63" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="K63" t="s">
         <v>5</v>
       </c>
       <c r="L63" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M63" t="s">
         <v>6</v>
@@ -3900,7 +3891,7 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C64" s="2">
         <v>1</v>
@@ -3909,28 +3900,28 @@
         <v>0</v>
       </c>
       <c r="E64" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F64" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="G64" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H64" s="3">
-        <v>46176</v>
+        <v>46204</v>
       </c>
       <c r="I64" s="3">
-        <v>46182</v>
+        <v>46204</v>
       </c>
       <c r="J64" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K64" t="s">
         <v>5</v>
       </c>
       <c r="L64" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M64" t="s">
         <v>6</v>
@@ -3950,7 +3941,7 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C65" s="2">
         <v>1</v>
@@ -3959,28 +3950,28 @@
         <v>0</v>
       </c>
       <c r="E65" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F65" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G65" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="H65" s="3">
-        <v>46176</v>
+        <v>46199</v>
       </c>
       <c r="I65" s="3">
-        <v>46182</v>
+        <v>46204</v>
       </c>
       <c r="J65" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="K65" t="s">
         <v>5</v>
       </c>
       <c r="L65" s="3">
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="M65" t="s">
         <v>6</v>
@@ -4000,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C66" s="2">
         <v>1</v>
@@ -4009,19 +4000,19 @@
         <v>0</v>
       </c>
       <c r="E66" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F66" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="G66" s="3">
-        <v>46142</v>
+        <v>46148</v>
       </c>
       <c r="H66" s="3">
-        <v>46150</v>
+        <v>46279</v>
       </c>
       <c r="I66" s="3">
-        <v>46154</v>
+        <v>46281</v>
       </c>
       <c r="J66" t="s">
         <v>30</v>
@@ -4030,7 +4021,7 @@
         <v>5</v>
       </c>
       <c r="L66" s="3">
-        <v>46142</v>
+        <v>46148</v>
       </c>
       <c r="M66" t="s">
         <v>6</v>
@@ -4050,7 +4041,7 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C67" s="2">
         <v>1</v>
@@ -4059,19 +4050,19 @@
         <v>0</v>
       </c>
       <c r="E67" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="F67" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="G67" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="H67" s="3">
-        <v>46150</v>
+        <v>46183</v>
       </c>
       <c r="I67" s="3">
-        <v>46154</v>
+        <v>46189</v>
       </c>
       <c r="J67" t="s">
         <v>4</v>
@@ -4080,7 +4071,7 @@
         <v>5</v>
       </c>
       <c r="L67" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="M67" t="s">
         <v>6</v>
@@ -4100,7 +4091,7 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="C68" s="2">
         <v>1</v>
@@ -4109,19 +4100,19 @@
         <v>0</v>
       </c>
       <c r="E68" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="F68" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="G68" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="H68" s="3">
-        <v>46150</v>
+        <v>46237</v>
       </c>
       <c r="I68" s="3">
-        <v>46154</v>
+        <v>46255</v>
       </c>
       <c r="J68" t="s">
         <v>4</v>
@@ -4130,7 +4121,7 @@
         <v>5</v>
       </c>
       <c r="L68" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="M68" t="s">
         <v>6</v>
@@ -4150,7 +4141,7 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="C69" s="2">
         <v>1</v>
@@ -4159,28 +4150,28 @@
         <v>0</v>
       </c>
       <c r="E69" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="F69" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="G69" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="H69" s="3">
-        <v>46184</v>
+        <v>46153</v>
       </c>
       <c r="I69" s="3">
-        <v>46188</v>
+        <v>46156</v>
       </c>
       <c r="J69" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="K69" t="s">
         <v>5</v>
       </c>
       <c r="L69" s="3">
-        <v>46142</v>
+        <v>46153</v>
       </c>
       <c r="M69" t="s">
         <v>6</v>
@@ -4200,7 +4191,7 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="C70" s="2">
         <v>1</v>
@@ -4209,28 +4200,28 @@
         <v>0</v>
       </c>
       <c r="E70" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="F70" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="G70" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="H70" s="3">
-        <v>46184</v>
+        <v>46191</v>
       </c>
       <c r="I70" s="3">
-        <v>46188</v>
+        <v>46203</v>
       </c>
       <c r="J70" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="K70" t="s">
         <v>5</v>
       </c>
       <c r="L70" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="M70" t="s">
         <v>6</v>
@@ -4250,7 +4241,7 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="C71" s="2">
         <v>1</v>
@@ -4259,19 +4250,19 @@
         <v>0</v>
       </c>
       <c r="E71" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="F71" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="G71" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="H71" s="3">
         <v>46184</v>
       </c>
       <c r="I71" s="3">
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="J71" t="s">
         <v>4</v>
@@ -4280,7 +4271,7 @@
         <v>5</v>
       </c>
       <c r="L71" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="M71" t="s">
         <v>6</v>
@@ -4300,7 +4291,7 @@
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="C72" s="2">
         <v>1</v>
@@ -4309,28 +4300,28 @@
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>96</v>
+        <v>164</v>
       </c>
       <c r="F72" t="s">
-        <v>97</v>
+        <v>165</v>
       </c>
       <c r="G72" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="H72" s="3">
-        <v>46142</v>
+        <v>46240</v>
       </c>
       <c r="I72" s="3">
-        <v>46149</v>
+        <v>46265</v>
       </c>
       <c r="J72" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="K72" t="s">
         <v>5</v>
       </c>
       <c r="L72" s="3">
-        <v>46142</v>
+        <v>46154</v>
       </c>
       <c r="M72" t="s">
         <v>6</v>
@@ -4350,7 +4341,7 @@
         <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="C73" s="2">
         <v>1</v>
@@ -4359,28 +4350,28 @@
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>96</v>
+        <v>167</v>
       </c>
       <c r="F73" t="s">
-        <v>97</v>
+        <v>168</v>
       </c>
       <c r="G73" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="H73" s="3">
-        <v>46142</v>
+        <v>46209</v>
       </c>
       <c r="I73" s="3">
-        <v>46149</v>
+        <v>46211</v>
       </c>
       <c r="J73" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="K73" t="s">
         <v>5</v>
       </c>
       <c r="L73" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="M73" t="s">
         <v>6</v>
@@ -4400,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="C74" s="2">
         <v>1</v>
@@ -4409,28 +4400,28 @@
         <v>0</v>
       </c>
       <c r="E74" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="F74" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="G74" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="H74" s="3">
-        <v>46142</v>
+        <v>46203</v>
       </c>
       <c r="I74" s="3">
-        <v>46149</v>
+        <v>46206</v>
       </c>
       <c r="J74" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="K74" t="s">
         <v>5</v>
       </c>
       <c r="L74" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="M74" t="s">
         <v>6</v>
@@ -4450,7 +4441,7 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="C75" s="2">
         <v>1</v>
@@ -4459,19 +4450,19 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>96</v>
+        <v>122</v>
       </c>
       <c r="F75" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="G75" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="H75" s="3">
-        <v>46177</v>
+        <v>46336</v>
       </c>
       <c r="I75" s="3">
-        <v>46183</v>
+        <v>46338</v>
       </c>
       <c r="J75" t="s">
         <v>30</v>
@@ -4480,7 +4471,7 @@
         <v>5</v>
       </c>
       <c r="L75" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="M75" t="s">
         <v>6</v>
@@ -4500,7 +4491,7 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="C76" s="2">
         <v>1</v>
@@ -4509,28 +4500,28 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>96</v>
+        <v>122</v>
       </c>
       <c r="F76" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="G76" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="H76" s="3">
-        <v>46177</v>
+        <v>46336</v>
       </c>
       <c r="I76" s="3">
-        <v>46183</v>
+        <v>46338</v>
       </c>
       <c r="J76" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K76" t="s">
         <v>5</v>
       </c>
       <c r="L76" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="M76" t="s">
         <v>6</v>
@@ -4550,7 +4541,7 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C77" s="2">
         <v>1</v>
@@ -4559,28 +4550,28 @@
         <v>0</v>
       </c>
       <c r="E77" t="s">
-        <v>96</v>
+        <v>173</v>
       </c>
       <c r="F77" t="s">
-        <v>97</v>
+        <v>174</v>
       </c>
       <c r="G77" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="H77" s="3">
-        <v>46177</v>
+        <v>46164</v>
       </c>
       <c r="I77" s="3">
-        <v>46183</v>
+        <v>46168</v>
       </c>
       <c r="J77" t="s">
-        <v>30</v>
+        <v>175</v>
       </c>
       <c r="K77" t="s">
         <v>5</v>
       </c>
       <c r="L77" s="3">
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="M77" t="s">
         <v>6</v>
@@ -4600,7 +4591,7 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="C78" s="2">
         <v>1</v>
@@ -4609,28 +4600,28 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>153</v>
+        <v>177</v>
       </c>
       <c r="F78" t="s">
-        <v>154</v>
+        <v>178</v>
       </c>
       <c r="G78" s="3">
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="H78" s="3">
-        <v>46204</v>
+        <v>46157</v>
       </c>
       <c r="I78" s="3">
-        <v>46206</v>
+        <v>46162</v>
       </c>
       <c r="J78" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="K78" t="s">
         <v>5</v>
       </c>
       <c r="L78" s="3">
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="M78" t="s">
         <v>6</v>
@@ -4647,10 +4638,10 @@
     </row>
     <row r="79" spans="1:16">
       <c r="A79" t="s">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="B79" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="C79" s="2">
         <v>1</v>
@@ -4659,28 +4650,28 @@
         <v>0</v>
       </c>
       <c r="E79" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="F79" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="G79" s="3">
-        <v>46148</v>
+        <v>46043</v>
       </c>
       <c r="H79" s="3">
-        <v>46163</v>
+        <v>46051</v>
       </c>
       <c r="I79" s="3">
-        <v>46170</v>
+        <v>46057</v>
       </c>
       <c r="J79" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="K79" t="s">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="L79" s="3">
-        <v>46148</v>
+        <v>46043</v>
       </c>
       <c r="M79" t="s">
         <v>6</v>
@@ -4692,456 +4683,6 @@
         <v>8</v>
       </c>
       <c r="P79" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16">
-      <c r="A80" t="s">
-        <v>0</v>
-      </c>
-      <c r="B80" t="s">
-        <v>158</v>
-      </c>
-      <c r="C80" s="2">
-        <v>1</v>
-      </c>
-      <c r="D80" s="2">
-        <v>0</v>
-      </c>
-      <c r="E80" t="s">
-        <v>159</v>
-      </c>
-      <c r="F80" t="s">
-        <v>160</v>
-      </c>
-      <c r="G80" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H80" s="3">
-        <v>46157</v>
-      </c>
-      <c r="I80" s="3">
-        <v>46162</v>
-      </c>
-      <c r="J80" t="s">
-        <v>70</v>
-      </c>
-      <c r="K80" t="s">
-        <v>5</v>
-      </c>
-      <c r="L80" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M80" t="s">
-        <v>6</v>
-      </c>
-      <c r="N80" t="s">
-        <v>7</v>
-      </c>
-      <c r="O80" t="s">
-        <v>8</v>
-      </c>
-      <c r="P80" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16">
-      <c r="A81" t="s">
-        <v>0</v>
-      </c>
-      <c r="B81" t="s">
-        <v>161</v>
-      </c>
-      <c r="C81" s="2">
-        <v>1</v>
-      </c>
-      <c r="D81" s="2">
-        <v>0</v>
-      </c>
-      <c r="E81" t="s">
-        <v>162</v>
-      </c>
-      <c r="F81" t="s">
-        <v>163</v>
-      </c>
-      <c r="G81" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H81" s="3">
-        <v>46224</v>
-      </c>
-      <c r="I81" s="3">
-        <v>46262</v>
-      </c>
-      <c r="J81" t="s">
-        <v>30</v>
-      </c>
-      <c r="K81" t="s">
-        <v>5</v>
-      </c>
-      <c r="L81" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M81" t="s">
-        <v>6</v>
-      </c>
-      <c r="N81" t="s">
-        <v>7</v>
-      </c>
-      <c r="O81" t="s">
-        <v>8</v>
-      </c>
-      <c r="P81" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="82" spans="1:16">
-      <c r="A82" t="s">
-        <v>0</v>
-      </c>
-      <c r="B82" t="s">
-        <v>164</v>
-      </c>
-      <c r="C82" s="2">
-        <v>1</v>
-      </c>
-      <c r="D82" s="2">
-        <v>0</v>
-      </c>
-      <c r="E82" t="s">
-        <v>165</v>
-      </c>
-      <c r="F82" t="s">
-        <v>166</v>
-      </c>
-      <c r="G82" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H82" s="3">
-        <v>46212</v>
-      </c>
-      <c r="I82" s="3">
-        <v>46219</v>
-      </c>
-      <c r="J82" t="s">
-        <v>30</v>
-      </c>
-      <c r="K82" t="s">
-        <v>5</v>
-      </c>
-      <c r="L82" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M82" t="s">
-        <v>6</v>
-      </c>
-      <c r="N82" t="s">
-        <v>7</v>
-      </c>
-      <c r="O82" t="s">
-        <v>8</v>
-      </c>
-      <c r="P82" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="83" spans="1:16">
-      <c r="A83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B83" t="s">
-        <v>167</v>
-      </c>
-      <c r="C83" s="2">
-        <v>1</v>
-      </c>
-      <c r="D83" s="2">
-        <v>0</v>
-      </c>
-      <c r="E83" t="s">
-        <v>168</v>
-      </c>
-      <c r="F83" t="s">
-        <v>169</v>
-      </c>
-      <c r="G83" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H83" s="3">
-        <v>46197</v>
-      </c>
-      <c r="I83" s="3">
-        <v>46202</v>
-      </c>
-      <c r="J83" t="s">
-        <v>30</v>
-      </c>
-      <c r="K83" t="s">
-        <v>5</v>
-      </c>
-      <c r="L83" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M83" t="s">
-        <v>6</v>
-      </c>
-      <c r="N83" t="s">
-        <v>7</v>
-      </c>
-      <c r="O83" t="s">
-        <v>8</v>
-      </c>
-      <c r="P83" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="84" spans="1:16">
-      <c r="A84" t="s">
-        <v>0</v>
-      </c>
-      <c r="B84" t="s">
-        <v>170</v>
-      </c>
-      <c r="C84" s="2">
-        <v>1</v>
-      </c>
-      <c r="D84" s="2">
-        <v>0</v>
-      </c>
-      <c r="E84" t="s">
-        <v>171</v>
-      </c>
-      <c r="F84" t="s">
-        <v>172</v>
-      </c>
-      <c r="G84" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H84" s="3">
-        <v>46191</v>
-      </c>
-      <c r="I84" s="3">
-        <v>46197</v>
-      </c>
-      <c r="J84" t="s">
-        <v>30</v>
-      </c>
-      <c r="K84" t="s">
-        <v>5</v>
-      </c>
-      <c r="L84" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M84" t="s">
-        <v>6</v>
-      </c>
-      <c r="N84" t="s">
-        <v>7</v>
-      </c>
-      <c r="O84" t="s">
-        <v>8</v>
-      </c>
-      <c r="P84" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="85" spans="1:16">
-      <c r="A85" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" t="s">
-        <v>173</v>
-      </c>
-      <c r="C85" s="2">
-        <v>1</v>
-      </c>
-      <c r="D85" s="2">
-        <v>0</v>
-      </c>
-      <c r="E85" t="s">
-        <v>174</v>
-      </c>
-      <c r="F85" t="s">
-        <v>175</v>
-      </c>
-      <c r="G85" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H85" s="3">
-        <v>46204</v>
-      </c>
-      <c r="I85" s="3">
-        <v>46204</v>
-      </c>
-      <c r="J85" t="s">
-        <v>30</v>
-      </c>
-      <c r="K85" t="s">
-        <v>5</v>
-      </c>
-      <c r="L85" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M85" t="s">
-        <v>6</v>
-      </c>
-      <c r="N85" t="s">
-        <v>7</v>
-      </c>
-      <c r="O85" t="s">
-        <v>8</v>
-      </c>
-      <c r="P85" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16">
-      <c r="A86" t="s">
-        <v>0</v>
-      </c>
-      <c r="B86" t="s">
-        <v>176</v>
-      </c>
-      <c r="C86" s="2">
-        <v>1</v>
-      </c>
-      <c r="D86" s="2">
-        <v>0</v>
-      </c>
-      <c r="E86" t="s">
-        <v>177</v>
-      </c>
-      <c r="F86" t="s">
-        <v>178</v>
-      </c>
-      <c r="G86" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H86" s="3">
-        <v>46199</v>
-      </c>
-      <c r="I86" s="3">
-        <v>46204</v>
-      </c>
-      <c r="J86" t="s">
-        <v>30</v>
-      </c>
-      <c r="K86" t="s">
-        <v>5</v>
-      </c>
-      <c r="L86" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M86" t="s">
-        <v>6</v>
-      </c>
-      <c r="N86" t="s">
-        <v>7</v>
-      </c>
-      <c r="O86" t="s">
-        <v>8</v>
-      </c>
-      <c r="P86" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16">
-      <c r="A87" t="s">
-        <v>0</v>
-      </c>
-      <c r="B87" t="s">
-        <v>179</v>
-      </c>
-      <c r="C87" s="2">
-        <v>1</v>
-      </c>
-      <c r="D87" s="2">
-        <v>0</v>
-      </c>
-      <c r="E87" t="s">
-        <v>180</v>
-      </c>
-      <c r="F87" t="s">
-        <v>181</v>
-      </c>
-      <c r="G87" s="3">
-        <v>46148</v>
-      </c>
-      <c r="H87" s="3">
-        <v>46279</v>
-      </c>
-      <c r="I87" s="3">
-        <v>46281</v>
-      </c>
-      <c r="J87" t="s">
-        <v>30</v>
-      </c>
-      <c r="K87" t="s">
-        <v>5</v>
-      </c>
-      <c r="L87" s="3">
-        <v>46148</v>
-      </c>
-      <c r="M87" t="s">
-        <v>6</v>
-      </c>
-      <c r="N87" t="s">
-        <v>7</v>
-      </c>
-      <c r="O87" t="s">
-        <v>8</v>
-      </c>
-      <c r="P87" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16">
-      <c r="A88" t="s">
-        <v>182</v>
-      </c>
-      <c r="B88" t="s">
-        <v>183</v>
-      </c>
-      <c r="C88" s="2">
-        <v>1</v>
-      </c>
-      <c r="D88" s="2">
-        <v>0</v>
-      </c>
-      <c r="E88" t="s">
-        <v>184</v>
-      </c>
-      <c r="F88" t="s">
-        <v>185</v>
-      </c>
-      <c r="G88" s="3">
-        <v>46043</v>
-      </c>
-      <c r="H88" s="3">
-        <v>46051</v>
-      </c>
-      <c r="I88" s="3">
-        <v>46057</v>
-      </c>
-      <c r="J88" t="s">
-        <v>4</v>
-      </c>
-      <c r="K88" t="s">
-        <v>186</v>
-      </c>
-      <c r="L88" s="3">
-        <v>46043</v>
-      </c>
-      <c r="M88" t="s">
-        <v>6</v>
-      </c>
-      <c r="N88" t="s">
-        <v>7</v>
-      </c>
-      <c r="O88" t="s">
-        <v>8</v>
-      </c>
-      <c r="P88" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>